<commit_message>
Update: updated weekend times
</commit_message>
<xml_diff>
--- a/uploads/xlsx/Timetable Spring-26 (1st-8th) 1.6 (Updated Timetable).xlsx
+++ b/uploads/xlsx/Timetable Spring-26 (1st-8th) 1.6 (Updated Timetable).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\zPythonStuff\Superior Academic Tool\uploads\xlsx\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8396DD-FA8E-49A9-B00E-ED2644FBB723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B823D7C0-9253-4055-B586-61E74C1C6312}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17640" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="490" uniqueCount="340">
   <si>
     <t>Week</t>
   </si>
@@ -894,9 +894,6 @@
 Mr. Ansar Naseem</t>
   </si>
   <si>
-    <t xml:space="preserve">SE Auditorium </t>
-  </si>
-  <si>
     <t xml:space="preserve">Mobile Application Development 
 BSSE-6C
 Mr. Muhammad Aqib </t>
@@ -1344,15 +1341,6 @@
     <t xml:space="preserve">Ideology &amp; Constitution of Pakistan 
 BSSE-1A/BSDS-1A
 Mr. Ali Shan </t>
-  </si>
-  <si>
-    <t>08:00 -10:00</t>
-  </si>
-  <si>
-    <t>10:00 - 12:00</t>
-  </si>
-  <si>
-    <t>12:00 - 02:00</t>
   </si>
   <si>
     <t>Calculus &amp; Analytical Geometry 
@@ -1807,9 +1795,7 @@
     <font>
       <b/>
       <sz val="14"/>
-      <color theme="1"/>
       <name val="Arial"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="23">
@@ -3844,21 +3830,12 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="116" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="63" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="2" borderId="64" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3951,224 +3928,173 @@
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="68" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="85" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="16" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="12" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="6" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="81" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="22" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="7" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="125" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="47" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="96" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="14" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="132" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="15" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="21" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="11" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="8" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="12" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="121" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="7" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="19" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="12" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -4199,11 +4125,6 @@
     <xf numFmtId="0" fontId="12" fillId="2" borderId="104" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="57" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="44" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="107" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -4212,94 +4133,150 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="4" borderId="105" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="85" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="76" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="80" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="86" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="42" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="121" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="7" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="125" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="43" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="110" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="99" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="84" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="87" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="19" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="17" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="21" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="11" borderId="89" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="4" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="12" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="18" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="127" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="12" fillId="22" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="117" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    <xf numFmtId="0" fontId="13" fillId="20" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="8" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="49" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="132" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="111" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="40" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -4327,6 +4304,15 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="69" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="45" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="63" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="64" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="109" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -4576,10 +4562,10 @@
       <c r="D1" s="50"/>
       <c r="E1" s="50"/>
       <c r="F1" s="50"/>
-      <c r="G1" s="246"/>
-      <c r="H1" s="247"/>
-      <c r="I1" s="247"/>
-      <c r="J1" s="248"/>
+      <c r="G1" s="228"/>
+      <c r="H1" s="229"/>
+      <c r="I1" s="229"/>
+      <c r="J1" s="230"/>
       <c r="K1" s="51"/>
       <c r="L1" s="52"/>
       <c r="M1" s="52"/>
@@ -4600,20 +4586,20 @@
       <c r="AB1" s="53"/>
     </row>
     <row r="2" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="252" t="s">
-        <v>212</v>
-      </c>
-      <c r="B2" s="247"/>
-      <c r="C2" s="247"/>
-      <c r="D2" s="247"/>
-      <c r="E2" s="248"/>
+      <c r="A2" s="234" t="s">
+        <v>211</v>
+      </c>
+      <c r="B2" s="229"/>
+      <c r="C2" s="229"/>
+      <c r="D2" s="229"/>
+      <c r="E2" s="230"/>
       <c r="F2" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="G2" s="249"/>
-      <c r="H2" s="250"/>
-      <c r="I2" s="250"/>
-      <c r="J2" s="251"/>
+      <c r="G2" s="231"/>
+      <c r="H2" s="232"/>
+      <c r="I2" s="232"/>
+      <c r="J2" s="233"/>
       <c r="K2" s="55"/>
       <c r="L2" s="52"/>
       <c r="M2" s="52"/>
@@ -4634,18 +4620,18 @@
       <c r="AB2" s="53"/>
     </row>
     <row r="3" spans="1:28" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="253"/>
-      <c r="B3" s="254"/>
-      <c r="C3" s="254"/>
-      <c r="D3" s="254"/>
-      <c r="E3" s="255"/>
+      <c r="A3" s="235"/>
+      <c r="B3" s="236"/>
+      <c r="C3" s="236"/>
+      <c r="D3" s="236"/>
+      <c r="E3" s="237"/>
       <c r="F3" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="G3" s="259"/>
-      <c r="H3" s="260"/>
-      <c r="I3" s="260"/>
-      <c r="J3" s="261"/>
+      <c r="G3" s="241"/>
+      <c r="H3" s="242"/>
+      <c r="I3" s="242"/>
+      <c r="J3" s="243"/>
       <c r="K3" s="56"/>
       <c r="L3" s="52"/>
       <c r="M3" s="52"/>
@@ -4666,18 +4652,18 @@
       <c r="AB3" s="53"/>
     </row>
     <row r="4" spans="1:28" ht="16.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="256"/>
-      <c r="B4" s="257"/>
-      <c r="C4" s="257"/>
-      <c r="D4" s="257"/>
-      <c r="E4" s="258"/>
+      <c r="A4" s="238"/>
+      <c r="B4" s="239"/>
+      <c r="C4" s="239"/>
+      <c r="D4" s="239"/>
+      <c r="E4" s="240"/>
       <c r="F4" s="44" t="s">
         <v>0</v>
       </c>
-      <c r="G4" s="262"/>
-      <c r="H4" s="263"/>
-      <c r="I4" s="263"/>
-      <c r="J4" s="264"/>
+      <c r="G4" s="244"/>
+      <c r="H4" s="245"/>
+      <c r="I4" s="245"/>
+      <c r="J4" s="246"/>
       <c r="K4" s="57"/>
       <c r="L4" s="52"/>
       <c r="M4" s="52"/>
@@ -4703,29 +4689,29 @@
         <v>1</v>
       </c>
       <c r="C5" s="40"/>
-      <c r="D5" s="127" t="s">
+      <c r="D5" s="124" t="s">
+        <v>301</v>
+      </c>
+      <c r="E5" s="125" t="s">
+        <v>302</v>
+      </c>
+      <c r="F5" s="125" t="s">
+        <v>303</v>
+      </c>
+      <c r="G5" s="125" t="s">
+        <v>304</v>
+      </c>
+      <c r="H5" s="126" t="s">
         <v>305</v>
       </c>
-      <c r="E5" s="128" t="s">
+      <c r="I5" s="126" t="s">
         <v>306</v>
       </c>
-      <c r="F5" s="128" t="s">
+      <c r="J5" s="126" t="s">
         <v>307</v>
       </c>
-      <c r="G5" s="128" t="s">
+      <c r="K5" s="127" t="s">
         <v>308</v>
-      </c>
-      <c r="H5" s="129" t="s">
-        <v>309</v>
-      </c>
-      <c r="I5" s="129" t="s">
-        <v>310</v>
-      </c>
-      <c r="J5" s="129" t="s">
-        <v>311</v>
-      </c>
-      <c r="K5" s="130" t="s">
-        <v>312</v>
       </c>
       <c r="L5" s="52"/>
       <c r="M5" s="52"/>
@@ -4746,25 +4732,25 @@
       <c r="AB5" s="53"/>
     </row>
     <row r="6" spans="1:28" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="274" t="s">
+      <c r="A6" s="207" t="s">
         <v>1</v>
       </c>
       <c r="B6" s="114" t="s">
         <v>2</v>
       </c>
-      <c r="C6" s="265" t="s">
+      <c r="C6" s="247" t="s">
         <v>3</v>
       </c>
-      <c r="D6" s="271" t="s">
+      <c r="D6" s="250" t="s">
         <v>4</v>
       </c>
-      <c r="E6" s="272"/>
-      <c r="F6" s="272"/>
-      <c r="G6" s="270"/>
-      <c r="H6" s="269" t="s">
-        <v>323</v>
-      </c>
-      <c r="I6" s="270"/>
+      <c r="E6" s="251"/>
+      <c r="F6" s="251"/>
+      <c r="G6" s="249"/>
+      <c r="H6" s="248" t="s">
+        <v>319</v>
+      </c>
+      <c r="I6" s="249"/>
       <c r="J6" s="115"/>
       <c r="K6" s="116"/>
       <c r="L6" s="52"/>
@@ -4786,21 +4772,21 @@
       <c r="AB6" s="53"/>
     </row>
     <row r="7" spans="1:28" ht="65.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="275"/>
+      <c r="A7" s="208"/>
       <c r="B7" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="266"/>
-      <c r="D7" s="213" t="s">
+      <c r="C7" s="219"/>
+      <c r="D7" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="E7" s="168"/>
-      <c r="F7" s="168"/>
-      <c r="G7" s="161"/>
-      <c r="H7" s="215" t="s">
-        <v>278</v>
-      </c>
-      <c r="I7" s="161"/>
+      <c r="E7" s="175"/>
+      <c r="F7" s="175"/>
+      <c r="G7" s="168"/>
+      <c r="H7" s="181" t="s">
+        <v>274</v>
+      </c>
+      <c r="I7" s="168"/>
       <c r="J7" s="47"/>
       <c r="K7" s="117"/>
       <c r="L7" s="52"/>
@@ -4822,27 +4808,27 @@
       <c r="AB7" s="53"/>
     </row>
     <row r="8" spans="1:28" ht="46.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="275"/>
+      <c r="A8" s="208"/>
       <c r="B8" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="267" t="s">
+      <c r="C8" s="218" t="s">
         <v>7</v>
       </c>
-      <c r="D8" s="225" t="s">
-        <v>263</v>
-      </c>
-      <c r="E8" s="168"/>
+      <c r="D8" s="253" t="s">
+        <v>262</v>
+      </c>
+      <c r="E8" s="175"/>
       <c r="F8" s="178" t="s">
-        <v>214</v>
-      </c>
-      <c r="G8" s="161"/>
-      <c r="H8" s="163" t="s">
+        <v>213</v>
+      </c>
+      <c r="G8" s="168"/>
+      <c r="H8" s="256" t="s">
         <v>44</v>
       </c>
-      <c r="I8" s="164"/>
-      <c r="J8" s="230"/>
-      <c r="K8" s="273"/>
+      <c r="I8" s="177"/>
+      <c r="J8" s="186"/>
+      <c r="K8" s="213"/>
       <c r="L8" s="52"/>
       <c r="M8" s="52"/>
       <c r="N8" s="52"/>
@@ -4862,23 +4848,23 @@
       <c r="AB8" s="53"/>
     </row>
     <row r="9" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="275"/>
+      <c r="A9" s="208"/>
       <c r="B9" s="64" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="268"/>
-      <c r="D9" s="213" t="s">
+      <c r="C9" s="220"/>
+      <c r="D9" s="252" t="s">
         <v>10</v>
       </c>
-      <c r="E9" s="161"/>
-      <c r="F9" s="181" t="s">
+      <c r="E9" s="168"/>
+      <c r="F9" s="176" t="s">
         <v>11</v>
       </c>
-      <c r="G9" s="164"/>
-      <c r="H9" s="160" t="s">
+      <c r="G9" s="177"/>
+      <c r="H9" s="169" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="161"/>
+      <c r="I9" s="168"/>
       <c r="J9" s="62"/>
       <c r="K9" s="118"/>
       <c r="L9" s="52"/>
@@ -4900,23 +4886,23 @@
       <c r="AB9" s="53"/>
     </row>
     <row r="10" spans="1:28" ht="61.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="275"/>
+      <c r="A10" s="208"/>
       <c r="B10" s="31" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="268"/>
-      <c r="D10" s="225" t="s">
+      <c r="C10" s="220"/>
+      <c r="D10" s="253" t="s">
         <v>14</v>
       </c>
-      <c r="E10" s="161"/>
-      <c r="F10" s="196" t="s">
-        <v>321</v>
-      </c>
-      <c r="G10" s="161"/>
-      <c r="H10" s="162" t="s">
-        <v>220</v>
-      </c>
-      <c r="I10" s="161"/>
+      <c r="E10" s="168"/>
+      <c r="F10" s="254" t="s">
+        <v>317</v>
+      </c>
+      <c r="G10" s="168"/>
+      <c r="H10" s="199" t="s">
+        <v>219</v>
+      </c>
+      <c r="I10" s="168"/>
       <c r="J10" s="90"/>
       <c r="K10" s="118"/>
       <c r="L10" s="52"/>
@@ -4938,28 +4924,28 @@
       <c r="AB10" s="53"/>
     </row>
     <row r="11" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="275"/>
+      <c r="A11" s="208"/>
       <c r="B11" s="31" t="s">
         <v>15</v>
       </c>
-      <c r="C11" s="267" t="s">
+      <c r="C11" s="218" t="s">
         <v>16</v>
       </c>
-      <c r="D11" s="229" t="s">
+      <c r="D11" s="197" t="s">
         <v>17</v>
       </c>
-      <c r="E11" s="161"/>
+      <c r="E11" s="168"/>
       <c r="F11" s="178" t="s">
-        <v>262</v>
-      </c>
-      <c r="G11" s="161"/>
+        <v>261</v>
+      </c>
+      <c r="G11" s="168"/>
       <c r="H11" s="119" t="s">
         <v>18</v>
       </c>
-      <c r="I11" s="160" t="s">
+      <c r="I11" s="169" t="s">
         <v>19</v>
       </c>
-      <c r="J11" s="161"/>
+      <c r="J11" s="168"/>
       <c r="K11" s="120"/>
       <c r="L11" s="52"/>
       <c r="M11" s="52"/>
@@ -4980,24 +4966,24 @@
       <c r="AB11" s="53"/>
     </row>
     <row r="12" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="275"/>
+      <c r="A12" s="208"/>
       <c r="B12" s="31" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="268"/>
-      <c r="D12" s="173" t="s">
+      <c r="C12" s="220"/>
+      <c r="D12" s="167" t="s">
         <v>21</v>
       </c>
-      <c r="E12" s="161"/>
-      <c r="F12" s="160" t="s">
+      <c r="E12" s="168"/>
+      <c r="F12" s="169" t="s">
         <v>22</v>
       </c>
-      <c r="G12" s="161"/>
-      <c r="H12" s="174" t="s">
-        <v>228</v>
-      </c>
-      <c r="I12" s="161"/>
-      <c r="J12" s="181"/>
+      <c r="G12" s="168"/>
+      <c r="H12" s="198" t="s">
+        <v>227</v>
+      </c>
+      <c r="I12" s="168"/>
+      <c r="J12" s="176"/>
       <c r="K12" s="184"/>
       <c r="L12" s="52"/>
       <c r="M12" s="52"/>
@@ -5018,25 +5004,25 @@
       <c r="AB12" s="53"/>
     </row>
     <row r="13" spans="1:28" ht="87" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="275"/>
+      <c r="A13" s="208"/>
       <c r="B13" s="31" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="268"/>
-      <c r="D13" s="229" t="s">
-        <v>223</v>
-      </c>
-      <c r="E13" s="161"/>
-      <c r="F13" s="160" t="s">
+      <c r="C13" s="220"/>
+      <c r="D13" s="197" t="s">
+        <v>222</v>
+      </c>
+      <c r="E13" s="168"/>
+      <c r="F13" s="169" t="s">
         <v>24</v>
       </c>
-      <c r="G13" s="161"/>
-      <c r="H13" s="192" t="s">
-        <v>215</v>
-      </c>
-      <c r="I13" s="193"/>
-      <c r="J13" s="244"/>
-      <c r="K13" s="245"/>
+      <c r="G13" s="168"/>
+      <c r="H13" s="189" t="s">
+        <v>214</v>
+      </c>
+      <c r="I13" s="180"/>
+      <c r="J13" s="257"/>
+      <c r="K13" s="258"/>
       <c r="L13" s="52"/>
       <c r="M13" s="52"/>
       <c r="N13" s="52"/>
@@ -5056,24 +5042,24 @@
       <c r="AB13" s="53"/>
     </row>
     <row r="14" spans="1:28" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="275"/>
+      <c r="A14" s="208"/>
       <c r="B14" s="31" t="s">
         <v>25</v>
       </c>
-      <c r="C14" s="268"/>
-      <c r="D14" s="175" t="s">
+      <c r="C14" s="220"/>
+      <c r="D14" s="297" t="s">
         <v>26</v>
       </c>
-      <c r="E14" s="176"/>
-      <c r="F14" s="177" t="s">
-        <v>265</v>
-      </c>
-      <c r="G14" s="168"/>
-      <c r="H14" s="194" t="s">
+      <c r="E14" s="298"/>
+      <c r="F14" s="299" t="s">
+        <v>264</v>
+      </c>
+      <c r="G14" s="175"/>
+      <c r="H14" s="162" t="s">
         <v>27</v>
       </c>
-      <c r="I14" s="194"/>
-      <c r="J14" s="163" t="s">
+      <c r="I14" s="162"/>
+      <c r="J14" s="256" t="s">
         <v>8</v>
       </c>
       <c r="K14" s="184"/>
@@ -5096,24 +5082,24 @@
       <c r="AB14" s="53"/>
     </row>
     <row r="15" spans="1:28" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="275"/>
+      <c r="A15" s="208"/>
       <c r="B15" s="31" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="268"/>
-      <c r="D15" s="214" t="s">
-        <v>257</v>
-      </c>
-      <c r="E15" s="164"/>
+      <c r="C15" s="220"/>
+      <c r="D15" s="275" t="s">
+        <v>256</v>
+      </c>
+      <c r="E15" s="177"/>
       <c r="F15" s="178" t="s">
-        <v>279</v>
-      </c>
-      <c r="G15" s="161"/>
-      <c r="H15" s="179" t="s">
-        <v>242</v>
-      </c>
-      <c r="I15" s="164"/>
-      <c r="J15" s="181"/>
+        <v>275</v>
+      </c>
+      <c r="G15" s="168"/>
+      <c r="H15" s="300" t="s">
+        <v>241</v>
+      </c>
+      <c r="I15" s="177"/>
+      <c r="J15" s="176"/>
       <c r="K15" s="184"/>
       <c r="L15" s="52"/>
       <c r="M15" s="52"/>
@@ -5134,20 +5120,20 @@
       <c r="AB15" s="53"/>
     </row>
     <row r="16" spans="1:28" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="275"/>
+      <c r="A16" s="208"/>
       <c r="B16" s="31" t="s">
         <v>29</v>
       </c>
-      <c r="C16" s="268"/>
-      <c r="D16" s="180" t="s">
+      <c r="C16" s="220"/>
+      <c r="D16" s="301" t="s">
         <v>4</v>
       </c>
-      <c r="E16" s="161"/>
-      <c r="F16" s="181" t="s">
+      <c r="E16" s="168"/>
+      <c r="F16" s="176" t="s">
         <v>30</v>
       </c>
-      <c r="G16" s="164"/>
-      <c r="H16" s="182" t="s">
+      <c r="G16" s="177"/>
+      <c r="H16" s="188" t="s">
         <v>31</v>
       </c>
       <c r="I16" s="183"/>
@@ -5172,27 +5158,27 @@
       <c r="AB16" s="53"/>
     </row>
     <row r="17" spans="1:28" ht="71.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="275"/>
+      <c r="A17" s="208"/>
       <c r="B17" s="31" t="s">
         <v>32</v>
       </c>
-      <c r="C17" s="268"/>
-      <c r="D17" s="185" t="s">
-        <v>330</v>
-      </c>
-      <c r="E17" s="161"/>
-      <c r="F17" s="160" t="s">
+      <c r="C17" s="220"/>
+      <c r="D17" s="302" t="s">
+        <v>326</v>
+      </c>
+      <c r="E17" s="168"/>
+      <c r="F17" s="169" t="s">
         <v>33</v>
       </c>
-      <c r="G17" s="161"/>
-      <c r="H17" s="222" t="s">
-        <v>303</v>
-      </c>
-      <c r="I17" s="161"/>
-      <c r="J17" s="160" t="s">
+      <c r="G17" s="168"/>
+      <c r="H17" s="284" t="s">
+        <v>299</v>
+      </c>
+      <c r="I17" s="168"/>
+      <c r="J17" s="169" t="s">
         <v>34</v>
       </c>
-      <c r="K17" s="186"/>
+      <c r="K17" s="170"/>
       <c r="L17" s="52"/>
       <c r="M17" s="52"/>
       <c r="N17" s="52"/>
@@ -5212,27 +5198,27 @@
       <c r="AB17" s="53"/>
     </row>
     <row r="18" spans="1:28" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="275"/>
+      <c r="A18" s="208"/>
       <c r="B18" s="31" t="s">
         <v>35</v>
       </c>
-      <c r="C18" s="268"/>
-      <c r="D18" s="173" t="s">
-        <v>250</v>
-      </c>
-      <c r="E18" s="161"/>
-      <c r="F18" s="215" t="s">
-        <v>289</v>
-      </c>
-      <c r="G18" s="161"/>
-      <c r="H18" s="215" t="s">
+      <c r="C18" s="220"/>
+      <c r="D18" s="167" t="s">
+        <v>249</v>
+      </c>
+      <c r="E18" s="168"/>
+      <c r="F18" s="181" t="s">
+        <v>285</v>
+      </c>
+      <c r="G18" s="168"/>
+      <c r="H18" s="181" t="s">
         <v>37</v>
       </c>
-      <c r="I18" s="161"/>
-      <c r="J18" s="160" t="s">
+      <c r="I18" s="168"/>
+      <c r="J18" s="169" t="s">
         <v>38</v>
       </c>
-      <c r="K18" s="186"/>
+      <c r="K18" s="170"/>
       <c r="L18" s="52"/>
       <c r="M18" s="52"/>
       <c r="N18" s="52"/>
@@ -5252,23 +5238,23 @@
       <c r="AB18" s="53"/>
     </row>
     <row r="19" spans="1:28" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="275"/>
+      <c r="A19" s="208"/>
       <c r="B19" s="31" t="s">
         <v>39</v>
       </c>
-      <c r="C19" s="268"/>
-      <c r="D19" s="173" t="s">
+      <c r="C19" s="220"/>
+      <c r="D19" s="167" t="s">
         <v>40</v>
       </c>
-      <c r="E19" s="161"/>
-      <c r="F19" s="215" t="s">
-        <v>251</v>
-      </c>
-      <c r="G19" s="161"/>
-      <c r="H19" s="160" t="s">
+      <c r="E19" s="168"/>
+      <c r="F19" s="181" t="s">
+        <v>250</v>
+      </c>
+      <c r="G19" s="168"/>
+      <c r="H19" s="169" t="s">
         <v>41</v>
       </c>
-      <c r="I19" s="161"/>
+      <c r="I19" s="168"/>
       <c r="J19" s="60"/>
       <c r="K19" s="82"/>
       <c r="L19" s="52"/>
@@ -5290,23 +5276,23 @@
       <c r="AB19" s="53"/>
     </row>
     <row r="20" spans="1:28" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="276"/>
-      <c r="B20" s="121" t="s">
+      <c r="A20" s="209"/>
+      <c r="B20" s="323" t="s">
         <v>42</v>
       </c>
-      <c r="C20" s="277"/>
-      <c r="D20" s="216" t="s">
+      <c r="C20" s="255"/>
+      <c r="D20" s="172" t="s">
         <v>43</v>
       </c>
-      <c r="E20" s="212"/>
-      <c r="F20" s="216" t="s">
-        <v>213</v>
-      </c>
-      <c r="G20" s="212"/>
-      <c r="H20" s="217" t="s">
-        <v>301</v>
-      </c>
-      <c r="I20" s="212"/>
+      <c r="E20" s="166"/>
+      <c r="F20" s="172" t="s">
+        <v>212</v>
+      </c>
+      <c r="G20" s="166"/>
+      <c r="H20" s="276" t="s">
+        <v>297</v>
+      </c>
+      <c r="I20" s="166"/>
       <c r="J20" s="85"/>
       <c r="K20" s="86"/>
       <c r="L20" s="52"/>
@@ -5329,10 +5315,10 @@
     </row>
     <row r="21" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="73"/>
-      <c r="B21" s="278" t="s">
+      <c r="B21" s="216" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="190"/>
+      <c r="C21" s="217"/>
       <c r="D21" s="74"/>
       <c r="E21" s="87"/>
       <c r="F21" s="87"/>
@@ -5360,36 +5346,36 @@
       <c r="AB21" s="53"/>
     </row>
     <row r="22" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="274" t="s">
+      <c r="A22" s="207" t="s">
         <v>45</v>
       </c>
-      <c r="B22" s="150" t="s">
+      <c r="B22" s="147" t="s">
         <v>46</v>
       </c>
-      <c r="C22" s="151"/>
-      <c r="D22" s="152" t="s">
+      <c r="C22" s="148"/>
+      <c r="D22" s="149" t="s">
+        <v>301</v>
+      </c>
+      <c r="E22" s="131" t="s">
+        <v>302</v>
+      </c>
+      <c r="F22" s="131" t="s">
+        <v>303</v>
+      </c>
+      <c r="G22" s="131" t="s">
+        <v>304</v>
+      </c>
+      <c r="H22" s="150" t="s">
         <v>305</v>
       </c>
-      <c r="E22" s="134" t="s">
+      <c r="I22" s="150" t="s">
         <v>306</v>
       </c>
-      <c r="F22" s="134" t="s">
+      <c r="J22" s="150" t="s">
         <v>307</v>
       </c>
-      <c r="G22" s="134" t="s">
+      <c r="K22" s="151" t="s">
         <v>308</v>
-      </c>
-      <c r="H22" s="153" t="s">
-        <v>309</v>
-      </c>
-      <c r="I22" s="153" t="s">
-        <v>310</v>
-      </c>
-      <c r="J22" s="153" t="s">
-        <v>311</v>
-      </c>
-      <c r="K22" s="154" t="s">
-        <v>312</v>
       </c>
       <c r="L22" s="52"/>
       <c r="M22" s="52"/>
@@ -5410,23 +5396,23 @@
       <c r="AB22" s="53"/>
     </row>
     <row r="23" spans="1:28" ht="42" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="275"/>
+      <c r="A23" s="208"/>
       <c r="B23" s="41" t="s">
         <v>47</v>
       </c>
-      <c r="C23" s="267" t="s">
+      <c r="C23" s="218" t="s">
         <v>3</v>
       </c>
-      <c r="D23" s="200" t="s">
+      <c r="D23" s="279" t="s">
         <v>4</v>
       </c>
-      <c r="E23" s="201"/>
-      <c r="F23" s="201"/>
-      <c r="G23" s="202"/>
-      <c r="H23" s="203" t="s">
-        <v>239</v>
-      </c>
-      <c r="I23" s="202"/>
+      <c r="E23" s="280"/>
+      <c r="F23" s="280"/>
+      <c r="G23" s="281"/>
+      <c r="H23" s="282" t="s">
+        <v>238</v>
+      </c>
+      <c r="I23" s="281"/>
       <c r="J23" s="58"/>
       <c r="K23" s="97"/>
       <c r="L23" s="52"/>
@@ -5448,21 +5434,21 @@
       <c r="AB23" s="53"/>
     </row>
     <row r="24" spans="1:28" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A24" s="275"/>
+      <c r="A24" s="208"/>
       <c r="B24" s="41" t="s">
         <v>48</v>
       </c>
-      <c r="C24" s="266"/>
-      <c r="D24" s="213" t="s">
+      <c r="C24" s="219"/>
+      <c r="D24" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="E24" s="168"/>
-      <c r="F24" s="168"/>
-      <c r="G24" s="161"/>
-      <c r="H24" s="221" t="s">
+      <c r="E24" s="175"/>
+      <c r="F24" s="175"/>
+      <c r="G24" s="168"/>
+      <c r="H24" s="283" t="s">
         <v>49</v>
       </c>
-      <c r="I24" s="164"/>
+      <c r="I24" s="177"/>
       <c r="J24" s="46"/>
       <c r="K24" s="98"/>
       <c r="L24" s="52"/>
@@ -5484,27 +5470,27 @@
       <c r="AB24" s="53"/>
     </row>
     <row r="25" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="275"/>
+      <c r="A25" s="208"/>
       <c r="B25" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C25" s="267" t="s">
+      <c r="C25" s="218" t="s">
         <v>7</v>
       </c>
-      <c r="D25" s="189" t="s">
-        <v>264</v>
-      </c>
-      <c r="E25" s="190"/>
-      <c r="F25" s="192" t="s">
-        <v>244</v>
-      </c>
-      <c r="G25" s="193"/>
-      <c r="H25" s="160" t="s">
+      <c r="D25" s="288" t="s">
+        <v>263</v>
+      </c>
+      <c r="E25" s="217"/>
+      <c r="F25" s="189" t="s">
+        <v>243</v>
+      </c>
+      <c r="G25" s="180"/>
+      <c r="H25" s="169" t="s">
         <v>50</v>
       </c>
-      <c r="I25" s="161"/>
-      <c r="J25" s="160"/>
-      <c r="K25" s="186"/>
+      <c r="I25" s="168"/>
+      <c r="J25" s="169"/>
+      <c r="K25" s="170"/>
       <c r="L25" s="52"/>
       <c r="M25" s="52"/>
       <c r="N25" s="52"/>
@@ -5524,25 +5510,25 @@
       <c r="AB25" s="53"/>
     </row>
     <row r="26" spans="1:28" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="275"/>
+      <c r="A26" s="208"/>
       <c r="B26" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C26" s="268"/>
-      <c r="D26" s="162" t="s">
-        <v>288</v>
-      </c>
-      <c r="E26" s="168"/>
-      <c r="F26" s="191" t="s">
+      <c r="C26" s="220"/>
+      <c r="D26" s="199" t="s">
+        <v>284</v>
+      </c>
+      <c r="E26" s="175"/>
+      <c r="F26" s="289" t="s">
         <v>51</v>
       </c>
-      <c r="G26" s="172"/>
-      <c r="H26" s="163" t="s">
+      <c r="G26" s="195"/>
+      <c r="H26" s="256" t="s">
         <v>52</v>
       </c>
-      <c r="I26" s="164"/>
-      <c r="J26" s="160"/>
-      <c r="K26" s="186"/>
+      <c r="I26" s="177"/>
+      <c r="J26" s="169"/>
+      <c r="K26" s="170"/>
       <c r="L26" s="52"/>
       <c r="M26" s="52"/>
       <c r="N26" s="52"/>
@@ -5562,25 +5548,25 @@
       <c r="AB26" s="53"/>
     </row>
     <row r="27" spans="1:28" ht="54.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="275"/>
+      <c r="A27" s="208"/>
       <c r="B27" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C27" s="266"/>
-      <c r="D27" s="229" t="s">
-        <v>249</v>
-      </c>
-      <c r="E27" s="168"/>
-      <c r="F27" s="230" t="s">
+      <c r="C27" s="219"/>
+      <c r="D27" s="197" t="s">
+        <v>248</v>
+      </c>
+      <c r="E27" s="175"/>
+      <c r="F27" s="186" t="s">
         <v>54</v>
       </c>
-      <c r="G27" s="198"/>
-      <c r="H27" s="160" t="s">
+      <c r="G27" s="187"/>
+      <c r="H27" s="169" t="s">
         <v>55</v>
       </c>
-      <c r="I27" s="161"/>
-      <c r="J27" s="160"/>
-      <c r="K27" s="186"/>
+      <c r="I27" s="168"/>
+      <c r="J27" s="169"/>
+      <c r="K27" s="170"/>
       <c r="L27" s="52"/>
       <c r="M27" s="52"/>
       <c r="N27" s="52"/>
@@ -5600,25 +5586,25 @@
       <c r="AB27" s="53"/>
     </row>
     <row r="28" spans="1:28" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="275"/>
+      <c r="A28" s="208"/>
       <c r="B28" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C28" s="279" t="s">
+      <c r="C28" s="221" t="s">
         <v>16</v>
       </c>
-      <c r="D28" s="227" t="s">
-        <v>331</v>
-      </c>
-      <c r="E28" s="219"/>
-      <c r="F28" s="231" t="s">
-        <v>284</v>
-      </c>
-      <c r="G28" s="161"/>
-      <c r="H28" s="160" t="s">
+      <c r="D28" s="270" t="s">
+        <v>327</v>
+      </c>
+      <c r="E28" s="271"/>
+      <c r="F28" s="174" t="s">
+        <v>280</v>
+      </c>
+      <c r="G28" s="168"/>
+      <c r="H28" s="169" t="s">
         <v>63</v>
       </c>
-      <c r="I28" s="161"/>
+      <c r="I28" s="168"/>
       <c r="J28" s="63"/>
       <c r="K28" s="118"/>
       <c r="L28" s="52"/>
@@ -5640,27 +5626,27 @@
       <c r="AB28" s="53"/>
     </row>
     <row r="29" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="275"/>
+      <c r="A29" s="208"/>
       <c r="B29" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C29" s="280"/>
-      <c r="D29" s="208" t="s">
-        <v>229</v>
-      </c>
-      <c r="E29" s="161"/>
-      <c r="F29" s="232" t="s">
-        <v>261</v>
-      </c>
-      <c r="G29" s="161"/>
-      <c r="H29" s="197" t="s">
+      <c r="C29" s="222"/>
+      <c r="D29" s="303" t="s">
+        <v>228</v>
+      </c>
+      <c r="E29" s="168"/>
+      <c r="F29" s="272" t="s">
+        <v>260</v>
+      </c>
+      <c r="G29" s="168"/>
+      <c r="H29" s="290" t="s">
         <v>56</v>
       </c>
-      <c r="I29" s="198"/>
-      <c r="J29" s="160" t="s">
+      <c r="I29" s="187"/>
+      <c r="J29" s="169" t="s">
         <v>57</v>
       </c>
-      <c r="K29" s="186"/>
+      <c r="K29" s="170"/>
       <c r="L29" s="52"/>
       <c r="M29" s="52"/>
       <c r="N29" s="52"/>
@@ -5680,23 +5666,23 @@
       <c r="AB29" s="53"/>
     </row>
     <row r="30" spans="1:28" ht="47.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="275"/>
+      <c r="A30" s="208"/>
       <c r="B30" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C30" s="280"/>
-      <c r="D30" s="173" t="s">
+      <c r="C30" s="222"/>
+      <c r="D30" s="167" t="s">
         <v>58</v>
       </c>
-      <c r="E30" s="161"/>
-      <c r="F30" s="223" t="s">
-        <v>255</v>
-      </c>
-      <c r="G30" s="224"/>
-      <c r="H30" s="207" t="s">
-        <v>280</v>
-      </c>
-      <c r="I30" s="161"/>
+      <c r="E30" s="168"/>
+      <c r="F30" s="267" t="s">
+        <v>254</v>
+      </c>
+      <c r="G30" s="268"/>
+      <c r="H30" s="273" t="s">
+        <v>276</v>
+      </c>
+      <c r="I30" s="168"/>
       <c r="J30" s="35"/>
       <c r="K30" s="118"/>
       <c r="L30" s="52"/>
@@ -5718,24 +5704,24 @@
       <c r="AB30" s="53"/>
     </row>
     <row r="31" spans="1:28" ht="62.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="275"/>
+      <c r="A31" s="208"/>
       <c r="B31" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C31" s="280"/>
-      <c r="D31" s="173" t="s">
+      <c r="C31" s="222"/>
+      <c r="D31" s="167" t="s">
         <v>59</v>
       </c>
-      <c r="E31" s="161"/>
-      <c r="F31" s="228" t="s">
+      <c r="E31" s="168"/>
+      <c r="F31" s="215" t="s">
         <v>60</v>
       </c>
-      <c r="G31" s="193"/>
+      <c r="G31" s="180"/>
       <c r="H31" s="63"/>
-      <c r="I31" s="181" t="s">
+      <c r="I31" s="176" t="s">
         <v>61</v>
       </c>
-      <c r="J31" s="164"/>
+      <c r="J31" s="177"/>
       <c r="K31" s="99"/>
       <c r="L31" s="52"/>
       <c r="M31" s="52"/>
@@ -5756,27 +5742,27 @@
       <c r="AB31" s="53"/>
     </row>
     <row r="32" spans="1:28" ht="66.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="275"/>
+      <c r="A32" s="208"/>
       <c r="B32" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C32" s="280"/>
-      <c r="D32" s="173" t="s">
+      <c r="C32" s="222"/>
+      <c r="D32" s="167" t="s">
         <v>62</v>
       </c>
-      <c r="E32" s="168"/>
-      <c r="F32" s="169" t="s">
-        <v>324</v>
-      </c>
-      <c r="G32" s="170"/>
-      <c r="H32" s="173" t="s">
+      <c r="E32" s="175"/>
+      <c r="F32" s="295" t="s">
+        <v>320</v>
+      </c>
+      <c r="G32" s="296"/>
+      <c r="H32" s="167" t="s">
         <v>64</v>
       </c>
-      <c r="I32" s="161"/>
-      <c r="J32" s="173" t="s">
+      <c r="I32" s="168"/>
+      <c r="J32" s="167" t="s">
         <v>65</v>
       </c>
-      <c r="K32" s="186"/>
+      <c r="K32" s="170"/>
       <c r="L32" s="52"/>
       <c r="M32" s="52"/>
       <c r="N32" s="52"/>
@@ -5796,24 +5782,24 @@
       <c r="AB32" s="53"/>
     </row>
     <row r="33" spans="1:28" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="275"/>
+      <c r="A33" s="208"/>
       <c r="B33" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C33" s="280"/>
-      <c r="D33" s="215" t="s">
+      <c r="C33" s="222"/>
+      <c r="D33" s="181" t="s">
         <v>66</v>
       </c>
-      <c r="E33" s="161"/>
-      <c r="F33" s="204" t="s">
+      <c r="E33" s="168"/>
+      <c r="F33" s="291" t="s">
         <v>4</v>
       </c>
-      <c r="G33" s="164"/>
-      <c r="H33" s="220" t="s">
+      <c r="G33" s="177"/>
+      <c r="H33" s="278" t="s">
         <v>4</v>
       </c>
-      <c r="I33" s="161"/>
-      <c r="J33" s="163"/>
+      <c r="I33" s="168"/>
+      <c r="J33" s="256"/>
       <c r="K33" s="184"/>
       <c r="L33" s="52"/>
       <c r="M33" s="52"/>
@@ -5834,25 +5820,25 @@
       <c r="AB33" s="53"/>
     </row>
     <row r="34" spans="1:28" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="275"/>
+      <c r="A34" s="208"/>
       <c r="B34" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C34" s="280"/>
-      <c r="D34" s="218" t="s">
-        <v>252</v>
-      </c>
-      <c r="E34" s="219"/>
-      <c r="F34" s="196" t="s">
-        <v>325</v>
-      </c>
-      <c r="G34" s="161"/>
-      <c r="H34" s="197" t="s">
+      <c r="C34" s="222"/>
+      <c r="D34" s="277" t="s">
+        <v>251</v>
+      </c>
+      <c r="E34" s="271"/>
+      <c r="F34" s="254" t="s">
+        <v>321</v>
+      </c>
+      <c r="G34" s="168"/>
+      <c r="H34" s="290" t="s">
         <v>67</v>
       </c>
-      <c r="I34" s="198"/>
-      <c r="J34" s="192"/>
-      <c r="K34" s="199"/>
+      <c r="I34" s="187"/>
+      <c r="J34" s="189"/>
+      <c r="K34" s="203"/>
       <c r="L34" s="52"/>
       <c r="M34" s="52"/>
       <c r="N34" s="52"/>
@@ -5872,25 +5858,25 @@
       <c r="AB34" s="53"/>
     </row>
     <row r="35" spans="1:28" ht="54.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="275"/>
+      <c r="A35" s="208"/>
       <c r="B35" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="281"/>
-      <c r="D35" s="207" t="s">
-        <v>221</v>
-      </c>
-      <c r="E35" s="161"/>
-      <c r="F35" s="205" t="s">
-        <v>332</v>
+      <c r="C35" s="223"/>
+      <c r="D35" s="273" t="s">
+        <v>220</v>
+      </c>
+      <c r="E35" s="168"/>
+      <c r="F35" s="292" t="s">
+        <v>328</v>
       </c>
       <c r="G35" s="183"/>
-      <c r="H35" s="160" t="s">
+      <c r="H35" s="169" t="s">
         <v>68</v>
       </c>
-      <c r="I35" s="161"/>
-      <c r="J35" s="206"/>
-      <c r="K35" s="199"/>
+      <c r="I35" s="168"/>
+      <c r="J35" s="202"/>
+      <c r="K35" s="203"/>
       <c r="L35" s="52"/>
       <c r="M35" s="52"/>
       <c r="N35" s="52"/>
@@ -5910,27 +5896,27 @@
       <c r="AB35" s="53"/>
     </row>
     <row r="36" spans="1:28" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A36" s="275"/>
+      <c r="A36" s="208"/>
       <c r="B36" s="32" t="s">
         <v>39</v>
       </c>
       <c r="C36" s="33" t="s">
         <v>7</v>
       </c>
-      <c r="D36" s="173" t="s">
+      <c r="D36" s="167" t="s">
         <v>69</v>
       </c>
-      <c r="E36" s="161"/>
-      <c r="F36" s="215" t="s">
+      <c r="E36" s="168"/>
+      <c r="F36" s="181" t="s">
         <v>36</v>
       </c>
-      <c r="G36" s="161"/>
-      <c r="H36" s="233" t="s">
-        <v>285</v>
-      </c>
-      <c r="I36" s="164"/>
-      <c r="J36" s="158"/>
-      <c r="K36" s="159"/>
+      <c r="G36" s="168"/>
+      <c r="H36" s="285" t="s">
+        <v>281</v>
+      </c>
+      <c r="I36" s="177"/>
+      <c r="J36" s="155"/>
+      <c r="K36" s="156"/>
       <c r="L36" s="52"/>
       <c r="M36" s="52"/>
       <c r="N36" s="52"/>
@@ -5950,26 +5936,26 @@
       <c r="AB36" s="53"/>
     </row>
     <row r="37" spans="1:28" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A37" s="276"/>
-      <c r="B37" s="122" t="s">
+      <c r="A37" s="209"/>
+      <c r="B37" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="C37" s="155" t="s">
+      <c r="C37" s="152" t="s">
         <v>16</v>
       </c>
-      <c r="D37" s="216" t="s">
+      <c r="D37" s="172" t="s">
         <v>70</v>
       </c>
-      <c r="E37" s="212"/>
-      <c r="F37" s="209" t="s">
+      <c r="E37" s="166"/>
+      <c r="F37" s="171" t="s">
         <v>71</v>
       </c>
-      <c r="G37" s="210"/>
-      <c r="H37" s="211" t="s">
-        <v>235</v>
-      </c>
-      <c r="I37" s="212"/>
-      <c r="J37" s="156"/>
+      <c r="G37" s="304"/>
+      <c r="H37" s="305" t="s">
+        <v>234</v>
+      </c>
+      <c r="I37" s="166"/>
+      <c r="J37" s="153"/>
       <c r="K37" s="103"/>
       <c r="L37" s="52"/>
       <c r="M37" s="52"/>
@@ -5991,10 +5977,10 @@
     </row>
     <row r="38" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="34"/>
-      <c r="B38" s="278" t="s">
+      <c r="B38" s="216" t="s">
         <v>72</v>
       </c>
-      <c r="C38" s="190"/>
+      <c r="C38" s="217"/>
       <c r="D38" s="74"/>
       <c r="E38" s="87"/>
       <c r="F38" s="87"/>
@@ -6022,36 +6008,36 @@
       <c r="AB38" s="53"/>
     </row>
     <row r="39" spans="1:28" ht="22.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A39" s="274" t="s">
+      <c r="A39" s="207" t="s">
         <v>72</v>
       </c>
       <c r="B39" s="95" t="s">
         <v>46</v>
       </c>
       <c r="C39" s="76"/>
-      <c r="D39" s="127" t="s">
+      <c r="D39" s="124" t="s">
+        <v>301</v>
+      </c>
+      <c r="E39" s="125" t="s">
+        <v>302</v>
+      </c>
+      <c r="F39" s="125" t="s">
+        <v>303</v>
+      </c>
+      <c r="G39" s="125" t="s">
+        <v>304</v>
+      </c>
+      <c r="H39" s="126" t="s">
         <v>305</v>
       </c>
-      <c r="E39" s="128" t="s">
+      <c r="I39" s="126" t="s">
         <v>306</v>
       </c>
-      <c r="F39" s="128" t="s">
+      <c r="J39" s="126" t="s">
         <v>307</v>
       </c>
-      <c r="G39" s="128" t="s">
+      <c r="K39" s="127" t="s">
         <v>308</v>
-      </c>
-      <c r="H39" s="129" t="s">
-        <v>309</v>
-      </c>
-      <c r="I39" s="129" t="s">
-        <v>310</v>
-      </c>
-      <c r="J39" s="129" t="s">
-        <v>311</v>
-      </c>
-      <c r="K39" s="130" t="s">
-        <v>312</v>
       </c>
       <c r="L39" s="52"/>
       <c r="M39" s="52"/>
@@ -6072,23 +6058,23 @@
       <c r="AB39" s="53"/>
     </row>
     <row r="40" spans="1:28" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="275"/>
+      <c r="A40" s="208"/>
       <c r="B40" s="41" t="s">
-        <v>269</v>
-      </c>
-      <c r="C40" s="267" t="s">
+        <v>268</v>
+      </c>
+      <c r="C40" s="218" t="s">
         <v>3</v>
       </c>
-      <c r="D40" s="200" t="s">
+      <c r="D40" s="279" t="s">
         <v>4</v>
       </c>
-      <c r="E40" s="201"/>
-      <c r="F40" s="201"/>
-      <c r="G40" s="202"/>
-      <c r="H40" s="203" t="s">
-        <v>281</v>
-      </c>
-      <c r="I40" s="202"/>
+      <c r="E40" s="280"/>
+      <c r="F40" s="280"/>
+      <c r="G40" s="281"/>
+      <c r="H40" s="282" t="s">
+        <v>277</v>
+      </c>
+      <c r="I40" s="281"/>
       <c r="J40" s="58"/>
       <c r="K40" s="97"/>
       <c r="L40" s="52"/>
@@ -6110,21 +6096,21 @@
       <c r="AB40" s="53"/>
     </row>
     <row r="41" spans="1:28" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A41" s="275"/>
+      <c r="A41" s="208"/>
       <c r="B41" s="41" t="s">
         <v>73</v>
       </c>
-      <c r="C41" s="266"/>
-      <c r="D41" s="213" t="s">
+      <c r="C41" s="219"/>
+      <c r="D41" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="E41" s="168"/>
-      <c r="F41" s="168"/>
-      <c r="G41" s="161"/>
-      <c r="H41" s="165" t="s">
+      <c r="E41" s="175"/>
+      <c r="F41" s="175"/>
+      <c r="G41" s="168"/>
+      <c r="H41" s="274" t="s">
         <v>75</v>
       </c>
-      <c r="I41" s="161"/>
+      <c r="I41" s="168"/>
       <c r="J41" s="92"/>
       <c r="K41" s="110"/>
       <c r="L41" s="52"/>
@@ -6146,21 +6132,21 @@
       <c r="AB41" s="53"/>
     </row>
     <row r="42" spans="1:28" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A42" s="275"/>
+      <c r="A42" s="208"/>
       <c r="B42" s="41" t="s">
         <v>74</v>
       </c>
       <c r="C42" s="59"/>
-      <c r="D42" s="213" t="s">
+      <c r="D42" s="252" t="s">
         <v>4</v>
       </c>
-      <c r="E42" s="168"/>
-      <c r="F42" s="226"/>
-      <c r="G42" s="193"/>
-      <c r="H42" s="165" t="s">
+      <c r="E42" s="175"/>
+      <c r="F42" s="269"/>
+      <c r="G42" s="180"/>
+      <c r="H42" s="274" t="s">
         <v>90</v>
       </c>
-      <c r="I42" s="166"/>
+      <c r="I42" s="293"/>
       <c r="J42" s="108"/>
       <c r="K42" s="109"/>
       <c r="L42" s="60"/>
@@ -6182,27 +6168,27 @@
       <c r="AB42" s="61"/>
     </row>
     <row r="43" spans="1:28" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="275"/>
+      <c r="A43" s="208"/>
       <c r="B43" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C43" s="267" t="s">
+      <c r="C43" s="218" t="s">
         <v>76</v>
       </c>
-      <c r="D43" s="229" t="s">
+      <c r="D43" s="197" t="s">
         <v>77</v>
       </c>
-      <c r="E43" s="168"/>
-      <c r="F43" s="291" t="s">
-        <v>326</v>
-      </c>
-      <c r="G43" s="172"/>
-      <c r="H43" s="163" t="s">
+      <c r="E43" s="175"/>
+      <c r="F43" s="161" t="s">
+        <v>322</v>
+      </c>
+      <c r="G43" s="195"/>
+      <c r="H43" s="256" t="s">
         <v>78</v>
       </c>
-      <c r="I43" s="164"/>
-      <c r="J43" s="289"/>
-      <c r="K43" s="273"/>
+      <c r="I43" s="177"/>
+      <c r="J43" s="212"/>
+      <c r="K43" s="213"/>
       <c r="L43" s="52"/>
       <c r="M43" s="52"/>
       <c r="N43" s="52"/>
@@ -6222,23 +6208,23 @@
       <c r="AB43" s="53"/>
     </row>
     <row r="44" spans="1:28" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="275"/>
+      <c r="A44" s="208"/>
       <c r="B44" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="C44" s="268"/>
-      <c r="D44" s="160" t="s">
+      <c r="C44" s="220"/>
+      <c r="D44" s="169" t="s">
         <v>89</v>
       </c>
-      <c r="E44" s="168"/>
-      <c r="F44" s="290" t="s">
-        <v>243</v>
-      </c>
-      <c r="G44" s="198"/>
-      <c r="H44" s="228" t="s">
-        <v>240</v>
-      </c>
-      <c r="I44" s="193"/>
+      <c r="E44" s="175"/>
+      <c r="F44" s="214" t="s">
+        <v>242</v>
+      </c>
+      <c r="G44" s="187"/>
+      <c r="H44" s="215" t="s">
+        <v>239</v>
+      </c>
+      <c r="I44" s="180"/>
       <c r="J44" s="35"/>
       <c r="K44" s="99"/>
       <c r="L44" s="52"/>
@@ -6260,25 +6246,25 @@
       <c r="AB44" s="53"/>
     </row>
     <row r="45" spans="1:28" ht="49.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A45" s="275"/>
+      <c r="A45" s="208"/>
       <c r="B45" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C45" s="266"/>
-      <c r="D45" s="286" t="s">
-        <v>245</v>
+      <c r="C45" s="219"/>
+      <c r="D45" s="201" t="s">
+        <v>244</v>
       </c>
       <c r="E45" s="183"/>
-      <c r="F45" s="236" t="s">
-        <v>260</v>
-      </c>
-      <c r="G45" s="172"/>
-      <c r="H45" s="171" t="s">
-        <v>234</v>
-      </c>
-      <c r="I45" s="172"/>
-      <c r="J45" s="206"/>
-      <c r="K45" s="199"/>
+      <c r="F45" s="194" t="s">
+        <v>259</v>
+      </c>
+      <c r="G45" s="195"/>
+      <c r="H45" s="196" t="s">
+        <v>233</v>
+      </c>
+      <c r="I45" s="195"/>
+      <c r="J45" s="202"/>
+      <c r="K45" s="203"/>
       <c r="L45" s="52"/>
       <c r="M45" s="52"/>
       <c r="N45" s="52"/>
@@ -6298,29 +6284,29 @@
       <c r="AB45" s="53"/>
     </row>
     <row r="46" spans="1:28" ht="48.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="275"/>
+      <c r="A46" s="208"/>
       <c r="B46" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C46" s="267" t="s">
+      <c r="C46" s="218" t="s">
         <v>16</v>
       </c>
-      <c r="D46" s="167" t="s">
-        <v>230</v>
-      </c>
-      <c r="E46" s="168"/>
-      <c r="F46" s="295" t="s">
-        <v>253</v>
-      </c>
-      <c r="G46" s="172"/>
-      <c r="H46" s="286" t="s">
-        <v>258</v>
-      </c>
-      <c r="I46" s="164"/>
-      <c r="J46" s="160" t="s">
+      <c r="D46" s="294" t="s">
+        <v>229</v>
+      </c>
+      <c r="E46" s="175"/>
+      <c r="F46" s="205" t="s">
+        <v>252</v>
+      </c>
+      <c r="G46" s="195"/>
+      <c r="H46" s="201" t="s">
+        <v>257</v>
+      </c>
+      <c r="I46" s="177"/>
+      <c r="J46" s="169" t="s">
         <v>81</v>
       </c>
-      <c r="K46" s="186"/>
+      <c r="K46" s="170"/>
       <c r="L46" s="52"/>
       <c r="M46" s="52"/>
       <c r="N46" s="52"/>
@@ -6340,23 +6326,23 @@
       <c r="AB46" s="53"/>
     </row>
     <row r="47" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A47" s="275"/>
+      <c r="A47" s="208"/>
       <c r="B47" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C47" s="268"/>
-      <c r="D47" s="173" t="s">
+      <c r="C47" s="220"/>
+      <c r="D47" s="167" t="s">
         <v>82</v>
       </c>
-      <c r="E47" s="168"/>
-      <c r="F47" s="195" t="s">
-        <v>225</v>
-      </c>
-      <c r="G47" s="164"/>
-      <c r="H47" s="160" t="s">
+      <c r="E47" s="175"/>
+      <c r="F47" s="206" t="s">
+        <v>224</v>
+      </c>
+      <c r="G47" s="177"/>
+      <c r="H47" s="169" t="s">
         <v>83</v>
       </c>
-      <c r="I47" s="161"/>
+      <c r="I47" s="168"/>
       <c r="J47" s="65"/>
       <c r="K47" s="100"/>
       <c r="L47" s="52"/>
@@ -6378,25 +6364,25 @@
       <c r="AB47" s="53"/>
     </row>
     <row r="48" spans="1:28" ht="75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="275"/>
+      <c r="A48" s="208"/>
       <c r="B48" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C48" s="268"/>
-      <c r="D48" s="162" t="s">
+      <c r="C48" s="220"/>
+      <c r="D48" s="199" t="s">
         <v>80</v>
       </c>
-      <c r="E48" s="161"/>
-      <c r="F48" s="294" t="s">
-        <v>246</v>
-      </c>
-      <c r="G48" s="193"/>
-      <c r="H48" s="192" t="s">
-        <v>216</v>
-      </c>
-      <c r="I48" s="193"/>
-      <c r="J48" s="192"/>
-      <c r="K48" s="186"/>
+      <c r="E48" s="168"/>
+      <c r="F48" s="204" t="s">
+        <v>245</v>
+      </c>
+      <c r="G48" s="180"/>
+      <c r="H48" s="189" t="s">
+        <v>215</v>
+      </c>
+      <c r="I48" s="180"/>
+      <c r="J48" s="189"/>
+      <c r="K48" s="170"/>
       <c r="L48" s="52"/>
       <c r="M48" s="52"/>
       <c r="N48" s="52"/>
@@ -6416,26 +6402,26 @@
       <c r="AB48" s="53"/>
     </row>
     <row r="49" spans="1:28" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="275"/>
+      <c r="A49" s="208"/>
       <c r="B49" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C49" s="268"/>
-      <c r="D49" s="162" t="s">
+      <c r="C49" s="220"/>
+      <c r="D49" s="199" t="s">
         <v>84</v>
       </c>
-      <c r="E49" s="168"/>
+      <c r="E49" s="175"/>
       <c r="F49" s="88" t="s">
         <v>18</v>
       </c>
-      <c r="G49" s="194" t="s">
+      <c r="G49" s="162" t="s">
         <v>85</v>
       </c>
-      <c r="H49" s="172"/>
-      <c r="I49" s="292" t="s">
+      <c r="H49" s="195"/>
+      <c r="I49" s="266" t="s">
         <v>86</v>
       </c>
-      <c r="J49" s="172"/>
+      <c r="J49" s="195"/>
       <c r="K49" s="101"/>
       <c r="L49" s="52"/>
       <c r="M49" s="52"/>
@@ -6456,13 +6442,13 @@
       <c r="AB49" s="53"/>
     </row>
     <row r="50" spans="1:28" ht="64.5" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="275"/>
+      <c r="A50" s="208"/>
       <c r="B50" s="32" t="s">
         <v>87</v>
       </c>
-      <c r="C50" s="268"/>
-      <c r="D50" s="173"/>
-      <c r="E50" s="168"/>
+      <c r="C50" s="220"/>
+      <c r="D50" s="167"/>
+      <c r="E50" s="175"/>
       <c r="F50" s="88"/>
       <c r="G50" s="89"/>
       <c r="H50" s="88"/>
@@ -6488,23 +6474,23 @@
       <c r="AB50" s="53"/>
     </row>
     <row r="51" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="275"/>
+      <c r="A51" s="208"/>
       <c r="B51" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C51" s="268"/>
-      <c r="D51" s="213" t="s">
+      <c r="C51" s="220"/>
+      <c r="D51" s="252" t="s">
         <v>88</v>
       </c>
-      <c r="E51" s="168"/>
-      <c r="F51" s="171" t="s">
-        <v>282</v>
-      </c>
-      <c r="G51" s="172"/>
-      <c r="H51" s="195" t="s">
-        <v>222</v>
-      </c>
-      <c r="I51" s="164"/>
+      <c r="E51" s="175"/>
+      <c r="F51" s="196" t="s">
+        <v>278</v>
+      </c>
+      <c r="G51" s="195"/>
+      <c r="H51" s="206" t="s">
+        <v>221</v>
+      </c>
+      <c r="I51" s="177"/>
       <c r="J51" s="49"/>
       <c r="K51" s="79"/>
       <c r="L51" s="52"/>
@@ -6526,23 +6512,23 @@
       <c r="AB51" s="53"/>
     </row>
     <row r="52" spans="1:28" ht="57.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="275"/>
+      <c r="A52" s="208"/>
       <c r="B52" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C52" s="268"/>
-      <c r="D52" s="173" t="s">
-        <v>254</v>
-      </c>
-      <c r="E52" s="168"/>
-      <c r="F52" s="182" t="s">
+      <c r="C52" s="220"/>
+      <c r="D52" s="167" t="s">
+        <v>253</v>
+      </c>
+      <c r="E52" s="175"/>
+      <c r="F52" s="188" t="s">
         <v>4</v>
       </c>
-      <c r="G52" s="164"/>
-      <c r="H52" s="182" t="s">
+      <c r="G52" s="177"/>
+      <c r="H52" s="188" t="s">
         <v>31</v>
       </c>
-      <c r="I52" s="164"/>
+      <c r="I52" s="177"/>
       <c r="J52" s="87"/>
       <c r="K52" s="102"/>
       <c r="L52" s="52"/>
@@ -6564,25 +6550,25 @@
       <c r="AB52" s="53"/>
     </row>
     <row r="53" spans="1:28" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="275"/>
+      <c r="A53" s="208"/>
       <c r="B53" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C53" s="268"/>
-      <c r="D53" s="162" t="s">
+      <c r="C53" s="220"/>
+      <c r="D53" s="199" t="s">
         <v>91</v>
       </c>
-      <c r="E53" s="161"/>
+      <c r="E53" s="168"/>
       <c r="F53" s="178" t="s">
         <v>92</v>
       </c>
-      <c r="G53" s="161"/>
-      <c r="H53" s="293" t="s">
+      <c r="G53" s="168"/>
+      <c r="H53" s="200" t="s">
         <v>93</v>
       </c>
-      <c r="I53" s="161"/>
-      <c r="J53" s="192"/>
-      <c r="K53" s="199"/>
+      <c r="I53" s="168"/>
+      <c r="J53" s="189"/>
+      <c r="K53" s="203"/>
       <c r="L53" s="52"/>
       <c r="M53" s="52"/>
       <c r="N53" s="52"/>
@@ -6602,23 +6588,23 @@
       <c r="AB53" s="53"/>
     </row>
     <row r="54" spans="1:28" ht="53.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A54" s="275"/>
+      <c r="A54" s="208"/>
       <c r="B54" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C54" s="266"/>
-      <c r="D54" s="229" t="s">
+      <c r="C54" s="219"/>
+      <c r="D54" s="197" t="s">
         <v>99</v>
       </c>
-      <c r="E54" s="161"/>
-      <c r="F54" s="174" t="s">
+      <c r="E54" s="168"/>
+      <c r="F54" s="198" t="s">
         <v>95</v>
       </c>
-      <c r="G54" s="161"/>
-      <c r="H54" s="215" t="s">
+      <c r="G54" s="168"/>
+      <c r="H54" s="181" t="s">
         <v>96</v>
       </c>
-      <c r="I54" s="161"/>
+      <c r="I54" s="168"/>
       <c r="J54" s="66"/>
       <c r="K54" s="81"/>
       <c r="L54" s="52"/>
@@ -6640,25 +6626,25 @@
       <c r="AB54" s="53"/>
     </row>
     <row r="55" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="275"/>
+      <c r="A55" s="208"/>
       <c r="B55" s="35" t="s">
         <v>39</v>
       </c>
       <c r="C55" s="36" t="s">
         <v>7</v>
       </c>
-      <c r="D55" s="160" t="s">
+      <c r="D55" s="169" t="s">
         <v>97</v>
       </c>
-      <c r="E55" s="161"/>
-      <c r="F55" s="160" t="s">
+      <c r="E55" s="168"/>
+      <c r="F55" s="169" t="s">
         <v>98</v>
       </c>
-      <c r="G55" s="161"/>
-      <c r="H55" s="192" t="s">
+      <c r="G55" s="168"/>
+      <c r="H55" s="189" t="s">
         <v>94</v>
       </c>
-      <c r="I55" s="193"/>
+      <c r="I55" s="180"/>
       <c r="J55" s="90"/>
       <c r="K55" s="81"/>
       <c r="L55" s="52"/>
@@ -6680,25 +6666,25 @@
       <c r="AB55" s="53"/>
     </row>
     <row r="56" spans="1:28" ht="59.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A56" s="276"/>
+      <c r="A56" s="209"/>
       <c r="B56" s="83" t="s">
         <v>42</v>
       </c>
       <c r="C56" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="D56" s="209" t="s">
+      <c r="D56" s="171" t="s">
         <v>100</v>
       </c>
-      <c r="E56" s="212"/>
-      <c r="F56" s="209" t="s">
+      <c r="E56" s="166"/>
+      <c r="F56" s="171" t="s">
         <v>101</v>
       </c>
-      <c r="G56" s="216"/>
-      <c r="H56" s="301" t="s">
-        <v>327</v>
-      </c>
-      <c r="I56" s="299"/>
+      <c r="G56" s="172"/>
+      <c r="H56" s="173" t="s">
+        <v>323</v>
+      </c>
+      <c r="I56" s="163"/>
       <c r="J56" s="104"/>
       <c r="K56" s="103"/>
       <c r="L56" s="52"/>
@@ -6721,10 +6707,10 @@
     </row>
     <row r="57" spans="1:28" ht="21.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A57" s="73"/>
-      <c r="B57" s="278" t="s">
+      <c r="B57" s="216" t="s">
         <v>102</v>
       </c>
-      <c r="C57" s="190"/>
+      <c r="C57" s="217"/>
       <c r="D57" s="74"/>
       <c r="E57" s="48"/>
       <c r="F57" s="48"/>
@@ -6752,36 +6738,36 @@
       <c r="AB57" s="53"/>
     </row>
     <row r="58" spans="1:28" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A58" s="274" t="s">
+      <c r="A58" s="207" t="s">
         <v>102</v>
       </c>
       <c r="B58" s="75" t="s">
         <v>46</v>
       </c>
       <c r="C58" s="96"/>
-      <c r="D58" s="131" t="s">
+      <c r="D58" s="128" t="s">
+        <v>301</v>
+      </c>
+      <c r="E58" s="129" t="s">
+        <v>302</v>
+      </c>
+      <c r="F58" s="129" t="s">
+        <v>303</v>
+      </c>
+      <c r="G58" s="129" t="s">
+        <v>304</v>
+      </c>
+      <c r="H58" s="145" t="s">
         <v>305</v>
       </c>
-      <c r="E58" s="132" t="s">
+      <c r="I58" s="145" t="s">
         <v>306</v>
       </c>
-      <c r="F58" s="132" t="s">
+      <c r="J58" s="145" t="s">
         <v>307</v>
       </c>
-      <c r="G58" s="132" t="s">
+      <c r="K58" s="146" t="s">
         <v>308</v>
-      </c>
-      <c r="H58" s="148" t="s">
-        <v>309</v>
-      </c>
-      <c r="I58" s="148" t="s">
-        <v>310</v>
-      </c>
-      <c r="J58" s="148" t="s">
-        <v>311</v>
-      </c>
-      <c r="K58" s="149" t="s">
-        <v>312</v>
       </c>
       <c r="L58" s="52"/>
       <c r="M58" s="52"/>
@@ -6802,21 +6788,21 @@
       <c r="AB58" s="53"/>
     </row>
     <row r="59" spans="1:28" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="275"/>
+      <c r="A59" s="208"/>
       <c r="B59" s="37" t="s">
         <v>103</v>
       </c>
       <c r="C59" s="38"/>
-      <c r="D59" s="182" t="s">
+      <c r="D59" s="188" t="s">
         <v>4</v>
       </c>
       <c r="E59" s="183"/>
       <c r="F59" s="183"/>
-      <c r="G59" s="164"/>
-      <c r="H59" s="181" t="s">
+      <c r="G59" s="177"/>
+      <c r="H59" s="176" t="s">
         <v>104</v>
       </c>
-      <c r="I59" s="164"/>
+      <c r="I59" s="177"/>
       <c r="J59" s="48"/>
       <c r="K59" s="78"/>
       <c r="L59" s="52"/>
@@ -6838,21 +6824,21 @@
       <c r="AB59" s="53"/>
     </row>
     <row r="60" spans="1:28" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A60" s="275"/>
+      <c r="A60" s="208"/>
       <c r="B60" s="37" t="s">
         <v>105</v>
       </c>
       <c r="C60" s="38"/>
-      <c r="D60" s="182" t="s">
+      <c r="D60" s="188" t="s">
         <v>4</v>
       </c>
       <c r="E60" s="183"/>
       <c r="F60" s="183"/>
-      <c r="G60" s="164"/>
-      <c r="H60" s="160" t="s">
+      <c r="G60" s="177"/>
+      <c r="H60" s="169" t="s">
         <v>106</v>
       </c>
-      <c r="I60" s="168"/>
+      <c r="I60" s="175"/>
       <c r="J60" s="93"/>
       <c r="K60" s="78"/>
       <c r="L60" s="52"/>
@@ -6874,25 +6860,25 @@
       <c r="AB60" s="53"/>
     </row>
     <row r="61" spans="1:28" ht="56.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="275"/>
+      <c r="A61" s="208"/>
       <c r="B61" s="37" t="s">
         <v>6</v>
       </c>
-      <c r="C61" s="285" t="s">
+      <c r="C61" s="227" t="s">
         <v>7</v>
       </c>
-      <c r="D61" s="181" t="s">
+      <c r="D61" s="176" t="s">
         <v>107</v>
       </c>
-      <c r="E61" s="164"/>
-      <c r="F61" s="181" t="s">
+      <c r="E61" s="177"/>
+      <c r="F61" s="176" t="s">
         <v>108</v>
       </c>
-      <c r="G61" s="164"/>
-      <c r="H61" s="230" t="s">
+      <c r="G61" s="177"/>
+      <c r="H61" s="186" t="s">
         <v>109</v>
       </c>
-      <c r="I61" s="198"/>
+      <c r="I61" s="187"/>
       <c r="J61" s="67"/>
       <c r="K61" s="79"/>
       <c r="L61" s="52"/>
@@ -6914,23 +6900,23 @@
       <c r="AB61" s="53"/>
     </row>
     <row r="62" spans="1:28" ht="60" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="275"/>
+      <c r="A62" s="208"/>
       <c r="B62" s="35" t="s">
         <v>9</v>
       </c>
-      <c r="C62" s="280"/>
+      <c r="C62" s="222"/>
       <c r="D62" s="178" t="s">
-        <v>283</v>
-      </c>
-      <c r="E62" s="161"/>
-      <c r="F62" s="160" t="s">
+        <v>279</v>
+      </c>
+      <c r="E62" s="168"/>
+      <c r="F62" s="169" t="s">
         <v>110</v>
       </c>
-      <c r="G62" s="173"/>
-      <c r="H62" s="194" t="s">
+      <c r="G62" s="167"/>
+      <c r="H62" s="162" t="s">
         <v>111</v>
       </c>
-      <c r="I62" s="194"/>
+      <c r="I62" s="162"/>
       <c r="J62" s="77"/>
       <c r="K62" s="80"/>
       <c r="L62" s="52"/>
@@ -6952,23 +6938,23 @@
       <c r="AB62" s="53"/>
     </row>
     <row r="63" spans="1:28" ht="67.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="275"/>
+      <c r="A63" s="208"/>
       <c r="B63" s="35" t="s">
         <v>13</v>
       </c>
-      <c r="C63" s="281"/>
+      <c r="C63" s="223"/>
       <c r="D63" s="178" t="s">
-        <v>226</v>
-      </c>
-      <c r="E63" s="161"/>
-      <c r="F63" s="160" t="s">
-        <v>302</v>
-      </c>
-      <c r="G63" s="168"/>
-      <c r="H63" s="194" t="s">
+        <v>225</v>
+      </c>
+      <c r="E63" s="168"/>
+      <c r="F63" s="169" t="s">
+        <v>298</v>
+      </c>
+      <c r="G63" s="175"/>
+      <c r="H63" s="162" t="s">
         <v>113</v>
       </c>
-      <c r="I63" s="194"/>
+      <c r="I63" s="162"/>
       <c r="J63" s="77"/>
       <c r="K63" s="81"/>
       <c r="L63" s="52"/>
@@ -6990,29 +6976,29 @@
       <c r="AB63" s="53"/>
     </row>
     <row r="64" spans="1:28" ht="54" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="275"/>
+      <c r="A64" s="208"/>
       <c r="B64" s="35" t="s">
         <v>15</v>
       </c>
-      <c r="C64" s="279" t="s">
+      <c r="C64" s="221" t="s">
         <v>16</v>
       </c>
-      <c r="D64" s="215" t="s">
-        <v>224</v>
-      </c>
-      <c r="E64" s="161"/>
-      <c r="F64" s="160" t="s">
-        <v>236</v>
-      </c>
-      <c r="G64" s="161"/>
-      <c r="H64" s="181" t="s">
+      <c r="D64" s="181" t="s">
+        <v>223</v>
+      </c>
+      <c r="E64" s="168"/>
+      <c r="F64" s="169" t="s">
+        <v>235</v>
+      </c>
+      <c r="G64" s="168"/>
+      <c r="H64" s="176" t="s">
         <v>114</v>
       </c>
-      <c r="I64" s="164"/>
-      <c r="J64" s="160" t="s">
+      <c r="I64" s="177"/>
+      <c r="J64" s="169" t="s">
         <v>115</v>
       </c>
-      <c r="K64" s="186"/>
+      <c r="K64" s="170"/>
       <c r="L64" s="52"/>
       <c r="M64" s="52"/>
       <c r="N64" s="52"/>
@@ -7032,27 +7018,27 @@
       <c r="AB64" s="53"/>
     </row>
     <row r="65" spans="1:28" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A65" s="275"/>
+      <c r="A65" s="208"/>
       <c r="B65" s="35" t="s">
         <v>20</v>
       </c>
-      <c r="C65" s="280"/>
-      <c r="D65" s="304" t="s">
-        <v>231</v>
-      </c>
-      <c r="E65" s="161"/>
-      <c r="F65" s="302" t="s">
+      <c r="C65" s="222"/>
+      <c r="D65" s="185" t="s">
+        <v>230</v>
+      </c>
+      <c r="E65" s="168"/>
+      <c r="F65" s="179" t="s">
         <v>112</v>
       </c>
-      <c r="G65" s="193"/>
-      <c r="H65" s="160" t="s">
+      <c r="G65" s="180"/>
+      <c r="H65" s="169" t="s">
         <v>116</v>
       </c>
-      <c r="I65" s="161"/>
-      <c r="J65" s="173" t="s">
+      <c r="I65" s="168"/>
+      <c r="J65" s="167" t="s">
         <v>119</v>
       </c>
-      <c r="K65" s="186"/>
+      <c r="K65" s="170"/>
       <c r="L65" s="52"/>
       <c r="M65" s="52"/>
       <c r="N65" s="52"/>
@@ -7072,29 +7058,29 @@
       <c r="AB65" s="53"/>
     </row>
     <row r="66" spans="1:28" ht="63.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="275"/>
+      <c r="A66" s="208"/>
       <c r="B66" s="35" t="s">
         <v>23</v>
       </c>
-      <c r="C66" s="280"/>
-      <c r="D66" s="157" t="s">
+      <c r="C66" s="222"/>
+      <c r="D66" s="154" t="s">
+        <v>270</v>
+      </c>
+      <c r="E66" s="154" t="s">
         <v>271</v>
       </c>
-      <c r="E66" s="157" t="s">
-        <v>272</v>
-      </c>
-      <c r="F66" s="171" t="s">
-        <v>247</v>
-      </c>
-      <c r="G66" s="172"/>
-      <c r="H66" s="173" t="s">
+      <c r="F66" s="196" t="s">
+        <v>246</v>
+      </c>
+      <c r="G66" s="195"/>
+      <c r="H66" s="167" t="s">
         <v>117</v>
       </c>
-      <c r="I66" s="161"/>
-      <c r="J66" s="160" t="s">
+      <c r="I66" s="168"/>
+      <c r="J66" s="169" t="s">
         <v>118</v>
       </c>
-      <c r="K66" s="186"/>
+      <c r="K66" s="170"/>
       <c r="L66" s="52"/>
       <c r="M66" s="52"/>
       <c r="N66" s="52"/>
@@ -7114,26 +7100,26 @@
       <c r="AB66" s="53"/>
     </row>
     <row r="67" spans="1:28" ht="78.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A67" s="275"/>
+      <c r="A67" s="208"/>
       <c r="B67" s="35" t="s">
         <v>25</v>
       </c>
-      <c r="C67" s="280"/>
-      <c r="D67" s="303" t="s">
-        <v>233</v>
+      <c r="C67" s="222"/>
+      <c r="D67" s="182" t="s">
+        <v>232</v>
       </c>
       <c r="E67" s="183"/>
       <c r="F67" s="42" t="s">
+        <v>272</v>
+      </c>
+      <c r="G67" s="91" t="s">
         <v>273</v>
       </c>
-      <c r="G67" s="91" t="s">
-        <v>274</v>
-      </c>
-      <c r="H67" s="231" t="s">
-        <v>232</v>
-      </c>
-      <c r="I67" s="161"/>
-      <c r="J67" s="181" t="s">
+      <c r="H67" s="174" t="s">
+        <v>231</v>
+      </c>
+      <c r="I67" s="168"/>
+      <c r="J67" s="176" t="s">
         <v>120</v>
       </c>
       <c r="K67" s="184"/>
@@ -7156,27 +7142,27 @@
       <c r="AB67" s="53"/>
     </row>
     <row r="68" spans="1:28" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="275"/>
+      <c r="A68" s="208"/>
       <c r="B68" s="35" t="s">
         <v>28</v>
       </c>
-      <c r="C68" s="280"/>
-      <c r="D68" s="181" t="s">
+      <c r="C68" s="222"/>
+      <c r="D68" s="176" t="s">
         <v>121</v>
       </c>
-      <c r="E68" s="164"/>
-      <c r="F68" s="240" t="s">
-        <v>259</v>
-      </c>
-      <c r="G68" s="164"/>
+      <c r="E68" s="177"/>
+      <c r="F68" s="265" t="s">
+        <v>258</v>
+      </c>
+      <c r="G68" s="177"/>
       <c r="H68" s="178" t="s">
-        <v>256</v>
-      </c>
-      <c r="I68" s="161"/>
-      <c r="J68" s="160" t="s">
+        <v>255</v>
+      </c>
+      <c r="I68" s="168"/>
+      <c r="J68" s="169" t="s">
         <v>122</v>
       </c>
-      <c r="K68" s="186"/>
+      <c r="K68" s="170"/>
       <c r="L68" s="52"/>
       <c r="M68" s="52"/>
       <c r="N68" s="52"/>
@@ -7196,23 +7182,23 @@
       <c r="AB68" s="53"/>
     </row>
     <row r="69" spans="1:28" ht="49.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="275"/>
+      <c r="A69" s="208"/>
       <c r="B69" s="35" t="s">
         <v>29</v>
       </c>
-      <c r="C69" s="281"/>
-      <c r="D69" s="160" t="s">
+      <c r="C69" s="223"/>
+      <c r="D69" s="169" t="s">
         <v>123</v>
       </c>
-      <c r="E69" s="161"/>
-      <c r="F69" s="160" t="s">
+      <c r="E69" s="168"/>
+      <c r="F69" s="169" t="s">
         <v>4</v>
       </c>
-      <c r="G69" s="161"/>
-      <c r="H69" s="160" t="s">
+      <c r="G69" s="168"/>
+      <c r="H69" s="169" t="s">
         <v>4</v>
       </c>
-      <c r="I69" s="161"/>
+      <c r="I69" s="168"/>
       <c r="J69" s="60"/>
       <c r="K69" s="82"/>
       <c r="L69" s="52"/>
@@ -7234,27 +7220,27 @@
       <c r="AB69" s="53"/>
     </row>
     <row r="70" spans="1:28" ht="53.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="275"/>
+      <c r="A70" s="208"/>
       <c r="B70" s="35" t="s">
         <v>32</v>
       </c>
-      <c r="C70" s="279" t="s">
+      <c r="C70" s="221" t="s">
         <v>16</v>
       </c>
-      <c r="D70" s="160" t="s">
-        <v>237</v>
-      </c>
-      <c r="E70" s="241"/>
-      <c r="F70" s="160" t="s">
-        <v>286</v>
-      </c>
-      <c r="G70" s="161"/>
-      <c r="H70" s="242" t="s">
+      <c r="D70" s="169" t="s">
+        <v>236</v>
+      </c>
+      <c r="E70" s="259"/>
+      <c r="F70" s="169" t="s">
+        <v>282</v>
+      </c>
+      <c r="G70" s="168"/>
+      <c r="H70" s="260" t="s">
         <v>125</v>
       </c>
-      <c r="I70" s="161"/>
-      <c r="J70" s="160"/>
-      <c r="K70" s="243"/>
+      <c r="I70" s="168"/>
+      <c r="J70" s="169"/>
+      <c r="K70" s="261"/>
       <c r="L70" s="52"/>
       <c r="M70" s="52"/>
       <c r="N70" s="52"/>
@@ -7274,25 +7260,25 @@
       <c r="AB70" s="53"/>
     </row>
     <row r="71" spans="1:28" ht="51" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="275"/>
+      <c r="A71" s="208"/>
       <c r="B71" s="35" t="s">
         <v>35</v>
       </c>
-      <c r="C71" s="281"/>
-      <c r="D71" s="229" t="s">
+      <c r="C71" s="223"/>
+      <c r="D71" s="197" t="s">
         <v>79</v>
       </c>
-      <c r="E71" s="168"/>
+      <c r="E71" s="175"/>
       <c r="F71" s="178" t="s">
         <v>126</v>
       </c>
-      <c r="G71" s="161"/>
-      <c r="H71" s="181" t="s">
+      <c r="G71" s="168"/>
+      <c r="H71" s="176" t="s">
         <v>127</v>
       </c>
-      <c r="I71" s="164"/>
-      <c r="J71" s="160"/>
-      <c r="K71" s="186"/>
+      <c r="I71" s="177"/>
+      <c r="J71" s="169"/>
+      <c r="K71" s="170"/>
       <c r="L71" s="52"/>
       <c r="M71" s="52"/>
       <c r="N71" s="52"/>
@@ -7312,25 +7298,25 @@
       <c r="AB71" s="53"/>
     </row>
     <row r="72" spans="1:28" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="275"/>
+      <c r="A72" s="208"/>
       <c r="B72" s="35" t="s">
         <v>39</v>
       </c>
       <c r="C72" s="39" t="s">
         <v>128</v>
       </c>
-      <c r="D72" s="160" t="s">
+      <c r="D72" s="169" t="s">
         <v>129</v>
       </c>
-      <c r="E72" s="161"/>
-      <c r="F72" s="160" t="s">
+      <c r="E72" s="168"/>
+      <c r="F72" s="169" t="s">
         <v>130</v>
       </c>
-      <c r="G72" s="161"/>
-      <c r="H72" s="160" t="s">
+      <c r="G72" s="168"/>
+      <c r="H72" s="169" t="s">
         <v>131</v>
       </c>
-      <c r="I72" s="161"/>
+      <c r="I72" s="168"/>
       <c r="J72" s="47"/>
       <c r="K72" s="81"/>
       <c r="L72" s="52"/>
@@ -7352,25 +7338,25 @@
       <c r="AB72" s="53"/>
     </row>
     <row r="73" spans="1:28" ht="53.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A73" s="276"/>
+      <c r="A73" s="209"/>
       <c r="B73" s="83" t="s">
         <v>42</v>
       </c>
       <c r="C73" s="84" t="s">
         <v>16</v>
       </c>
-      <c r="D73" s="300" t="s">
-        <v>241</v>
-      </c>
-      <c r="E73" s="212"/>
-      <c r="F73" s="288" t="s">
-        <v>322</v>
-      </c>
-      <c r="G73" s="212"/>
-      <c r="H73" s="209" t="s">
+      <c r="D73" s="165" t="s">
+        <v>240</v>
+      </c>
+      <c r="E73" s="166"/>
+      <c r="F73" s="211" t="s">
+        <v>318</v>
+      </c>
+      <c r="G73" s="166"/>
+      <c r="H73" s="171" t="s">
         <v>124</v>
       </c>
-      <c r="I73" s="234"/>
+      <c r="I73" s="262"/>
       <c r="J73" s="85"/>
       <c r="K73" s="86"/>
       <c r="L73" s="52"/>
@@ -7393,10 +7379,10 @@
     </row>
     <row r="74" spans="1:28" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A74" s="73"/>
-      <c r="B74" s="278" t="s">
+      <c r="B74" s="216" t="s">
         <v>132</v>
       </c>
-      <c r="C74" s="190"/>
+      <c r="C74" s="217"/>
       <c r="D74" s="74"/>
       <c r="E74" s="48"/>
       <c r="F74" s="48"/>
@@ -7424,36 +7410,36 @@
       <c r="AB74" s="53"/>
     </row>
     <row r="75" spans="1:28" ht="27" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="287" t="s">
+      <c r="A75" s="210" t="s">
         <v>133</v>
       </c>
-      <c r="B75" s="146" t="s">
+      <c r="B75" s="143" t="s">
         <v>46</v>
       </c>
-      <c r="C75" s="147"/>
-      <c r="D75" s="131" t="s">
-        <v>313</v>
-      </c>
-      <c r="E75" s="132" t="s">
+      <c r="C75" s="144"/>
+      <c r="D75" s="128" t="s">
+        <v>309</v>
+      </c>
+      <c r="E75" s="129" t="s">
+        <v>310</v>
+      </c>
+      <c r="F75" s="129" t="s">
+        <v>311</v>
+      </c>
+      <c r="G75" s="129" t="s">
+        <v>312</v>
+      </c>
+      <c r="H75" s="145" t="s">
+        <v>269</v>
+      </c>
+      <c r="I75" s="145" t="s">
         <v>314</v>
       </c>
-      <c r="F75" s="132" t="s">
+      <c r="J75" s="146" t="s">
         <v>315</v>
       </c>
-      <c r="G75" s="132" t="s">
+      <c r="K75" s="146" t="s">
         <v>316</v>
-      </c>
-      <c r="H75" s="148" t="s">
-        <v>270</v>
-      </c>
-      <c r="I75" s="148" t="s">
-        <v>318</v>
-      </c>
-      <c r="J75" s="149" t="s">
-        <v>319</v>
-      </c>
-      <c r="K75" s="149" t="s">
-        <v>320</v>
       </c>
       <c r="L75" s="52"/>
       <c r="M75" s="52"/>
@@ -7474,25 +7460,25 @@
       <c r="AB75" s="53"/>
     </row>
     <row r="76" spans="1:28" ht="73.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="275"/>
-      <c r="B76" s="141" t="s">
+      <c r="A76" s="208"/>
+      <c r="B76" s="138" t="s">
         <v>134</v>
       </c>
-      <c r="C76" s="142" t="s">
+      <c r="C76" s="139" t="s">
         <v>3</v>
       </c>
-      <c r="D76" s="237"/>
-      <c r="E76" s="238"/>
-      <c r="F76" s="296" t="s">
-        <v>266</v>
-      </c>
-      <c r="G76" s="238"/>
-      <c r="H76" s="305" t="s">
-        <v>317</v>
-      </c>
-      <c r="I76" s="143"/>
-      <c r="J76" s="144"/>
-      <c r="K76" s="145"/>
+      <c r="D76" s="264"/>
+      <c r="E76" s="191"/>
+      <c r="F76" s="190" t="s">
+        <v>265</v>
+      </c>
+      <c r="G76" s="191"/>
+      <c r="H76" s="157" t="s">
+        <v>313</v>
+      </c>
+      <c r="I76" s="140"/>
+      <c r="J76" s="141"/>
+      <c r="K76" s="142"/>
       <c r="L76" s="52"/>
       <c r="M76" s="52"/>
       <c r="N76" s="52"/>
@@ -7512,25 +7498,25 @@
       <c r="AB76" s="53"/>
     </row>
     <row r="77" spans="1:28" ht="73.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="275"/>
+      <c r="A77" s="208"/>
       <c r="B77" s="41" t="s">
         <v>135</v>
       </c>
       <c r="C77" s="111" t="s">
         <v>3</v>
       </c>
-      <c r="D77" s="239" t="s">
+      <c r="D77" s="164" t="s">
         <v>4</v>
       </c>
-      <c r="E77" s="172"/>
-      <c r="F77" s="172"/>
-      <c r="G77" s="172"/>
-      <c r="H77" s="306"/>
-      <c r="I77" s="308" t="s">
-        <v>248</v>
-      </c>
-      <c r="J77" s="308"/>
-      <c r="K77" s="136"/>
+      <c r="E77" s="195"/>
+      <c r="F77" s="195"/>
+      <c r="G77" s="195"/>
+      <c r="H77" s="158"/>
+      <c r="I77" s="160" t="s">
+        <v>247</v>
+      </c>
+      <c r="J77" s="160"/>
+      <c r="K77" s="133"/>
       <c r="L77" s="52"/>
       <c r="M77" s="52"/>
       <c r="N77" s="52"/>
@@ -7550,27 +7536,27 @@
       <c r="AB77" s="53"/>
     </row>
     <row r="78" spans="1:28" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A78" s="275"/>
+      <c r="A78" s="208"/>
       <c r="B78" s="41" t="s">
         <v>6</v>
       </c>
-      <c r="C78" s="282" t="s">
+      <c r="C78" s="224" t="s">
         <v>136</v>
       </c>
-      <c r="D78" s="236" t="s">
+      <c r="D78" s="194" t="s">
         <v>137</v>
       </c>
-      <c r="E78" s="172"/>
-      <c r="F78" s="194" t="s">
+      <c r="E78" s="195"/>
+      <c r="F78" s="162" t="s">
         <v>138</v>
       </c>
-      <c r="G78" s="172"/>
-      <c r="H78" s="306"/>
-      <c r="I78" s="308" t="s">
-        <v>219</v>
-      </c>
-      <c r="J78" s="308"/>
-      <c r="K78" s="136"/>
+      <c r="G78" s="195"/>
+      <c r="H78" s="158"/>
+      <c r="I78" s="160" t="s">
+        <v>218</v>
+      </c>
+      <c r="J78" s="160"/>
+      <c r="K78" s="133"/>
       <c r="L78" s="52"/>
       <c r="M78" s="52"/>
       <c r="N78" s="52"/>
@@ -7590,25 +7576,25 @@
       <c r="AB78" s="53"/>
     </row>
     <row r="79" spans="1:28" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A79" s="275"/>
+      <c r="A79" s="208"/>
       <c r="B79" s="41" t="s">
         <v>9</v>
       </c>
-      <c r="C79" s="283"/>
-      <c r="D79" s="194" t="s">
+      <c r="C79" s="225"/>
+      <c r="D79" s="162" t="s">
         <v>139</v>
       </c>
-      <c r="E79" s="172"/>
-      <c r="F79" s="171" t="s">
+      <c r="E79" s="195"/>
+      <c r="F79" s="196" t="s">
         <v>53</v>
       </c>
-      <c r="G79" s="172"/>
-      <c r="H79" s="306"/>
-      <c r="I79" s="194" t="s">
+      <c r="G79" s="195"/>
+      <c r="H79" s="158"/>
+      <c r="I79" s="162" t="s">
         <v>140</v>
       </c>
-      <c r="J79" s="194"/>
-      <c r="K79" s="137"/>
+      <c r="J79" s="162"/>
+      <c r="K79" s="134"/>
       <c r="L79" s="52"/>
       <c r="M79" s="52"/>
       <c r="N79" s="52"/>
@@ -7628,25 +7614,25 @@
       <c r="AB79" s="53"/>
     </row>
     <row r="80" spans="1:28" ht="52.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A80" s="275"/>
+      <c r="A80" s="208"/>
       <c r="B80" s="32" t="s">
         <v>13</v>
       </c>
-      <c r="C80" s="284"/>
-      <c r="D80" s="194" t="s">
+      <c r="C80" s="226"/>
+      <c r="D80" s="162" t="s">
         <v>141</v>
       </c>
-      <c r="E80" s="172"/>
-      <c r="F80" s="171" t="s">
-        <v>290</v>
-      </c>
-      <c r="G80" s="172"/>
-      <c r="H80" s="306"/>
-      <c r="I80" s="194" t="s">
+      <c r="E80" s="195"/>
+      <c r="F80" s="196" t="s">
+        <v>286</v>
+      </c>
+      <c r="G80" s="195"/>
+      <c r="H80" s="158"/>
+      <c r="I80" s="162" t="s">
         <v>142</v>
       </c>
-      <c r="J80" s="194"/>
-      <c r="K80" s="137"/>
+      <c r="J80" s="162"/>
+      <c r="K80" s="134"/>
       <c r="L80" s="52"/>
       <c r="M80" s="52"/>
       <c r="N80" s="52"/>
@@ -7666,27 +7652,27 @@
       <c r="AB80" s="53"/>
     </row>
     <row r="81" spans="1:28" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A81" s="275"/>
+      <c r="A81" s="208"/>
       <c r="B81" s="32" t="s">
         <v>15</v>
       </c>
-      <c r="C81" s="282" t="s">
+      <c r="C81" s="224" t="s">
         <v>16</v>
       </c>
-      <c r="D81" s="194" t="s">
+      <c r="D81" s="162" t="s">
         <v>143</v>
       </c>
-      <c r="E81" s="172"/>
-      <c r="F81" s="194" t="s">
+      <c r="E81" s="195"/>
+      <c r="F81" s="162" t="s">
+        <v>216</v>
+      </c>
+      <c r="G81" s="195"/>
+      <c r="H81" s="158"/>
+      <c r="I81" s="162" t="s">
         <v>217</v>
       </c>
-      <c r="G81" s="172"/>
-      <c r="H81" s="306"/>
-      <c r="I81" s="194" t="s">
-        <v>218</v>
-      </c>
-      <c r="J81" s="194"/>
-      <c r="K81" s="137"/>
+      <c r="J81" s="162"/>
+      <c r="K81" s="134"/>
       <c r="L81" s="52"/>
       <c r="M81" s="52"/>
       <c r="N81" s="52"/>
@@ -7706,25 +7692,25 @@
       <c r="AB81" s="53"/>
     </row>
     <row r="82" spans="1:28" ht="61.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A82" s="275"/>
+      <c r="A82" s="208"/>
       <c r="B82" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="C82" s="283"/>
-      <c r="D82" s="291" t="s">
-        <v>328</v>
-      </c>
-      <c r="E82" s="172"/>
-      <c r="F82" s="235" t="s">
-        <v>304</v>
-      </c>
-      <c r="G82" s="172"/>
-      <c r="H82" s="306"/>
-      <c r="I82" s="194" t="s">
+      <c r="C82" s="225"/>
+      <c r="D82" s="161" t="s">
+        <v>324</v>
+      </c>
+      <c r="E82" s="195"/>
+      <c r="F82" s="263" t="s">
+        <v>300</v>
+      </c>
+      <c r="G82" s="195"/>
+      <c r="H82" s="158"/>
+      <c r="I82" s="162" t="s">
         <v>144</v>
       </c>
-      <c r="J82" s="194"/>
-      <c r="K82" s="137"/>
+      <c r="J82" s="162"/>
+      <c r="K82" s="134"/>
       <c r="L82" s="52"/>
       <c r="M82" s="52"/>
       <c r="N82" s="52"/>
@@ -7744,25 +7730,25 @@
       <c r="AB82" s="53"/>
     </row>
     <row r="83" spans="1:28" ht="52.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A83" s="275"/>
+      <c r="A83" s="208"/>
       <c r="B83" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="C83" s="283"/>
-      <c r="D83" s="236" t="s">
-        <v>287</v>
-      </c>
-      <c r="E83" s="172"/>
-      <c r="F83" s="194" t="s">
+      <c r="C83" s="225"/>
+      <c r="D83" s="194" t="s">
+        <v>283</v>
+      </c>
+      <c r="E83" s="195"/>
+      <c r="F83" s="162" t="s">
         <v>145</v>
       </c>
-      <c r="G83" s="172"/>
-      <c r="H83" s="306"/>
-      <c r="I83" s="194" t="s">
+      <c r="G83" s="195"/>
+      <c r="H83" s="158"/>
+      <c r="I83" s="162" t="s">
         <v>146</v>
       </c>
-      <c r="J83" s="194"/>
-      <c r="K83" s="137"/>
+      <c r="J83" s="162"/>
+      <c r="K83" s="134"/>
       <c r="L83" s="52"/>
       <c r="M83" s="52"/>
       <c r="N83" s="52"/>
@@ -7782,25 +7768,25 @@
       <c r="AB83" s="53"/>
     </row>
     <row r="84" spans="1:28" ht="51.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A84" s="275"/>
+      <c r="A84" s="208"/>
       <c r="B84" s="32" t="s">
         <v>25</v>
       </c>
-      <c r="C84" s="283"/>
-      <c r="D84" s="171" t="s">
-        <v>238</v>
-      </c>
-      <c r="E84" s="172"/>
-      <c r="F84" s="236" t="s">
+      <c r="C84" s="225"/>
+      <c r="D84" s="196" t="s">
+        <v>237</v>
+      </c>
+      <c r="E84" s="195"/>
+      <c r="F84" s="194" t="s">
         <v>147</v>
       </c>
-      <c r="G84" s="172"/>
-      <c r="H84" s="306"/>
-      <c r="I84" s="194" t="s">
+      <c r="G84" s="195"/>
+      <c r="H84" s="158"/>
+      <c r="I84" s="162" t="s">
         <v>148</v>
       </c>
-      <c r="J84" s="194"/>
-      <c r="K84" s="137"/>
+      <c r="J84" s="162"/>
+      <c r="K84" s="134"/>
       <c r="L84" s="52"/>
       <c r="M84" s="52"/>
       <c r="N84" s="52"/>
@@ -7820,25 +7806,25 @@
       <c r="AB84" s="53"/>
     </row>
     <row r="85" spans="1:28" ht="63" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="275"/>
+      <c r="A85" s="208"/>
       <c r="B85" s="32" t="s">
         <v>28</v>
       </c>
-      <c r="C85" s="283"/>
-      <c r="D85" s="194" t="s">
-        <v>227</v>
-      </c>
-      <c r="E85" s="172"/>
-      <c r="F85" s="194" t="s">
+      <c r="C85" s="225"/>
+      <c r="D85" s="162" t="s">
+        <v>226</v>
+      </c>
+      <c r="E85" s="195"/>
+      <c r="F85" s="162" t="s">
         <v>149</v>
       </c>
-      <c r="G85" s="172"/>
-      <c r="H85" s="306"/>
-      <c r="I85" s="291" t="s">
-        <v>329</v>
-      </c>
-      <c r="J85" s="194"/>
-      <c r="K85" s="137"/>
+      <c r="G85" s="195"/>
+      <c r="H85" s="158"/>
+      <c r="I85" s="161" t="s">
+        <v>325</v>
+      </c>
+      <c r="J85" s="162"/>
+      <c r="K85" s="134"/>
       <c r="L85" s="52"/>
       <c r="M85" s="52"/>
       <c r="N85" s="52"/>
@@ -7858,25 +7844,25 @@
       <c r="AB85" s="53"/>
     </row>
     <row r="86" spans="1:28" ht="60.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A86" s="275"/>
+      <c r="A86" s="208"/>
       <c r="B86" s="32" t="s">
         <v>29</v>
       </c>
-      <c r="C86" s="283"/>
-      <c r="D86" s="194" t="s">
+      <c r="C86" s="225"/>
+      <c r="D86" s="162" t="s">
         <v>150</v>
       </c>
-      <c r="E86" s="172"/>
-      <c r="F86" s="239" t="s">
+      <c r="E86" s="195"/>
+      <c r="F86" s="164" t="s">
         <v>4</v>
       </c>
-      <c r="G86" s="172"/>
-      <c r="H86" s="306"/>
-      <c r="I86" s="239" t="s">
+      <c r="G86" s="195"/>
+      <c r="H86" s="158"/>
+      <c r="I86" s="164" t="s">
         <v>151</v>
       </c>
-      <c r="J86" s="239"/>
-      <c r="K86" s="138"/>
+      <c r="J86" s="164"/>
+      <c r="K86" s="135"/>
       <c r="L86" s="52"/>
       <c r="M86" s="52"/>
       <c r="N86" s="52"/>
@@ -7896,25 +7882,25 @@
       <c r="AB86" s="53"/>
     </row>
     <row r="87" spans="1:28" ht="45.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="275"/>
+      <c r="A87" s="208"/>
       <c r="B87" s="32" t="s">
         <v>32</v>
       </c>
-      <c r="C87" s="283"/>
-      <c r="D87" s="194" t="s">
+      <c r="C87" s="225"/>
+      <c r="D87" s="162" t="s">
         <v>152</v>
       </c>
-      <c r="E87" s="172"/>
-      <c r="F87" s="236" t="s">
+      <c r="E87" s="195"/>
+      <c r="F87" s="194" t="s">
         <v>153</v>
       </c>
-      <c r="G87" s="172"/>
-      <c r="H87" s="306"/>
-      <c r="I87" s="194" t="s">
+      <c r="G87" s="195"/>
+      <c r="H87" s="158"/>
+      <c r="I87" s="162" t="s">
         <v>154</v>
       </c>
-      <c r="J87" s="194"/>
-      <c r="K87" s="137"/>
+      <c r="J87" s="162"/>
+      <c r="K87" s="134"/>
       <c r="L87" s="52"/>
       <c r="M87" s="52"/>
       <c r="N87" s="52"/>
@@ -7934,19 +7920,19 @@
       <c r="AB87" s="53"/>
     </row>
     <row r="88" spans="1:28" ht="64.5" hidden="1" customHeight="1" x14ac:dyDescent="0.85">
-      <c r="A88" s="275"/>
+      <c r="A88" s="208"/>
       <c r="B88" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C88" s="283"/>
+      <c r="C88" s="225"/>
       <c r="D88" s="93"/>
       <c r="E88" s="93"/>
       <c r="F88" s="93"/>
       <c r="G88" s="93"/>
-      <c r="H88" s="306"/>
-      <c r="I88" s="135"/>
-      <c r="J88" s="123"/>
-      <c r="K88" s="139"/>
+      <c r="H88" s="158"/>
+      <c r="I88" s="132"/>
+      <c r="J88" s="122"/>
+      <c r="K88" s="136"/>
       <c r="L88" s="52"/>
       <c r="M88" s="52"/>
       <c r="N88" s="52"/>
@@ -7966,25 +7952,25 @@
       <c r="AB88" s="53"/>
     </row>
     <row r="89" spans="1:28" ht="58.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="275"/>
+      <c r="A89" s="208"/>
       <c r="B89" s="32" t="s">
         <v>35</v>
       </c>
-      <c r="C89" s="284"/>
-      <c r="D89" s="194" t="s">
+      <c r="C89" s="226"/>
+      <c r="D89" s="162" t="s">
         <v>155</v>
       </c>
-      <c r="E89" s="172"/>
-      <c r="F89" s="194" t="s">
+      <c r="E89" s="195"/>
+      <c r="F89" s="162" t="s">
         <v>156</v>
       </c>
-      <c r="G89" s="172"/>
-      <c r="H89" s="306"/>
-      <c r="I89" s="194" t="s">
+      <c r="G89" s="195"/>
+      <c r="H89" s="158"/>
+      <c r="I89" s="162" t="s">
         <v>157</v>
       </c>
-      <c r="J89" s="194"/>
-      <c r="K89" s="137"/>
+      <c r="J89" s="162"/>
+      <c r="K89" s="134"/>
       <c r="L89" s="52"/>
       <c r="M89" s="52"/>
       <c r="N89" s="52"/>
@@ -8004,27 +7990,27 @@
       <c r="AB89" s="53"/>
     </row>
     <row r="90" spans="1:28" ht="50.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="275"/>
+      <c r="A90" s="208"/>
       <c r="B90" s="32" t="s">
         <v>39</v>
       </c>
-      <c r="C90" s="133" t="s">
+      <c r="C90" s="130" t="s">
         <v>7</v>
       </c>
-      <c r="D90" s="194" t="s">
+      <c r="D90" s="162" t="s">
         <v>158</v>
       </c>
-      <c r="E90" s="172"/>
-      <c r="F90" s="194" t="s">
+      <c r="E90" s="195"/>
+      <c r="F90" s="162" t="s">
         <v>159</v>
       </c>
-      <c r="G90" s="172"/>
-      <c r="H90" s="306"/>
-      <c r="I90" s="194" t="s">
+      <c r="G90" s="195"/>
+      <c r="H90" s="158"/>
+      <c r="I90" s="162" t="s">
         <v>160</v>
       </c>
-      <c r="J90" s="194"/>
-      <c r="K90" s="137"/>
+      <c r="J90" s="162"/>
+      <c r="K90" s="134"/>
       <c r="L90" s="52"/>
       <c r="M90" s="52"/>
       <c r="N90" s="52"/>
@@ -8044,27 +8030,27 @@
       <c r="AB90" s="53"/>
     </row>
     <row r="91" spans="1:28" ht="46.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A91" s="276"/>
-      <c r="B91" s="122" t="s">
+      <c r="A91" s="209"/>
+      <c r="B91" s="121" t="s">
         <v>42</v>
       </c>
-      <c r="C91" s="124" t="s">
+      <c r="C91" s="123" t="s">
         <v>16</v>
       </c>
-      <c r="D91" s="297" t="s">
+      <c r="D91" s="192" t="s">
         <v>161</v>
       </c>
-      <c r="E91" s="298"/>
-      <c r="F91" s="299" t="s">
+      <c r="E91" s="193"/>
+      <c r="F91" s="163" t="s">
         <v>162</v>
       </c>
-      <c r="G91" s="298"/>
-      <c r="H91" s="307"/>
-      <c r="I91" s="299" t="s">
+      <c r="G91" s="193"/>
+      <c r="H91" s="159"/>
+      <c r="I91" s="163" t="s">
         <v>163</v>
       </c>
-      <c r="J91" s="299"/>
-      <c r="K91" s="140"/>
+      <c r="J91" s="163"/>
+      <c r="K91" s="137"/>
       <c r="L91" s="52"/>
       <c r="M91" s="52"/>
       <c r="N91" s="52"/>
@@ -8299,8 +8285,8 @@
       <c r="C99" s="68"/>
       <c r="D99" s="70"/>
       <c r="E99" s="70"/>
-      <c r="F99" s="187"/>
-      <c r="G99" s="188"/>
+      <c r="F99" s="286"/>
+      <c r="G99" s="287"/>
       <c r="H99" s="70"/>
       <c r="I99" s="70"/>
       <c r="J99" s="70"/>
@@ -35355,21 +35341,239 @@
     </row>
   </sheetData>
   <mergeCells count="272">
-    <mergeCell ref="H76:H91"/>
-    <mergeCell ref="I77:J77"/>
-    <mergeCell ref="I85:J85"/>
-    <mergeCell ref="I84:J84"/>
-    <mergeCell ref="I83:J83"/>
-    <mergeCell ref="I82:J82"/>
-    <mergeCell ref="I81:J81"/>
-    <mergeCell ref="I80:J80"/>
-    <mergeCell ref="I79:J79"/>
-    <mergeCell ref="I78:J78"/>
-    <mergeCell ref="I91:J91"/>
-    <mergeCell ref="I90:J90"/>
-    <mergeCell ref="I89:J89"/>
-    <mergeCell ref="I87:J87"/>
-    <mergeCell ref="I86:J86"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="H42:I42"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="F66:G66"/>
+    <mergeCell ref="F51:G51"/>
+    <mergeCell ref="F62:G62"/>
+    <mergeCell ref="H12:I12"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="F15:G15"/>
+    <mergeCell ref="H15:I15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="F16:G16"/>
+    <mergeCell ref="H16:K16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="F17:G17"/>
+    <mergeCell ref="J17:K17"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="F99:G99"/>
+    <mergeCell ref="H25:I25"/>
+    <mergeCell ref="J25:K25"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="F26:G26"/>
+    <mergeCell ref="H26:I26"/>
+    <mergeCell ref="J26:K26"/>
+    <mergeCell ref="F25:G25"/>
+    <mergeCell ref="H62:I62"/>
+    <mergeCell ref="H63:I63"/>
+    <mergeCell ref="H51:I51"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="D40:G40"/>
+    <mergeCell ref="H40:I40"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="F35:G35"/>
+    <mergeCell ref="H35:I35"/>
+    <mergeCell ref="J35:K35"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="D41:G41"/>
+    <mergeCell ref="H41:I41"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="F19:G19"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="D20:E20"/>
+    <mergeCell ref="F20:G20"/>
+    <mergeCell ref="H20:I20"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="J15:K15"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="H23:I23"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="H24:I24"/>
+    <mergeCell ref="H17:I17"/>
+    <mergeCell ref="H36:I36"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H43:I43"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H10:I10"/>
+    <mergeCell ref="D42:G42"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="I31:J31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="H28:I28"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="F28:G28"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="F36:G36"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J71:K71"/>
+    <mergeCell ref="D69:E69"/>
+    <mergeCell ref="F69:G69"/>
+    <mergeCell ref="D70:E70"/>
+    <mergeCell ref="F70:G70"/>
+    <mergeCell ref="H70:I70"/>
+    <mergeCell ref="J70:K70"/>
+    <mergeCell ref="F71:G71"/>
+    <mergeCell ref="J68:K68"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="H68:I68"/>
+    <mergeCell ref="F68:G68"/>
+    <mergeCell ref="H69:I69"/>
+    <mergeCell ref="H71:I71"/>
+    <mergeCell ref="H46:I46"/>
+    <mergeCell ref="H52:I52"/>
+    <mergeCell ref="D60:G60"/>
+    <mergeCell ref="D61:E61"/>
+    <mergeCell ref="D44:E44"/>
+    <mergeCell ref="D49:E49"/>
+    <mergeCell ref="G1:J2"/>
+    <mergeCell ref="A2:E4"/>
+    <mergeCell ref="G3:J3"/>
+    <mergeCell ref="G4:J4"/>
+    <mergeCell ref="C6:C7"/>
+    <mergeCell ref="C8:C10"/>
+    <mergeCell ref="H6:I6"/>
+    <mergeCell ref="D6:G6"/>
+    <mergeCell ref="D7:G7"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="J8:K8"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="A6:A20"/>
+    <mergeCell ref="C11:C20"/>
+    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="J12:K12"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="I11:J11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="B21:C21"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="C25:C27"/>
+    <mergeCell ref="C28:C35"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="C81:C89"/>
+    <mergeCell ref="C78:C80"/>
+    <mergeCell ref="C46:C54"/>
+    <mergeCell ref="C61:C63"/>
+    <mergeCell ref="C64:C69"/>
+    <mergeCell ref="B74:C74"/>
+    <mergeCell ref="B57:C57"/>
+    <mergeCell ref="C70:C71"/>
+    <mergeCell ref="C40:C41"/>
+    <mergeCell ref="C43:C45"/>
+    <mergeCell ref="H72:I72"/>
+    <mergeCell ref="F73:G73"/>
+    <mergeCell ref="J43:K43"/>
+    <mergeCell ref="D71:E71"/>
+    <mergeCell ref="F44:G44"/>
+    <mergeCell ref="H44:I44"/>
+    <mergeCell ref="D43:E43"/>
+    <mergeCell ref="F43:G43"/>
+    <mergeCell ref="D84:E84"/>
+    <mergeCell ref="D68:E68"/>
+    <mergeCell ref="F52:G52"/>
+    <mergeCell ref="H73:I73"/>
+    <mergeCell ref="F82:G82"/>
+    <mergeCell ref="D83:E83"/>
+    <mergeCell ref="F83:G83"/>
+    <mergeCell ref="D79:E79"/>
+    <mergeCell ref="D80:E80"/>
+    <mergeCell ref="D76:E76"/>
+    <mergeCell ref="D77:G77"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="D51:E51"/>
+    <mergeCell ref="J53:K53"/>
+    <mergeCell ref="A22:A37"/>
+    <mergeCell ref="A39:A56"/>
+    <mergeCell ref="A58:A73"/>
+    <mergeCell ref="A75:A91"/>
+    <mergeCell ref="D78:E78"/>
+    <mergeCell ref="F78:G78"/>
+    <mergeCell ref="F79:G79"/>
+    <mergeCell ref="D72:E72"/>
+    <mergeCell ref="F72:G72"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F64:G64"/>
+    <mergeCell ref="D48:E48"/>
+    <mergeCell ref="D54:E54"/>
+    <mergeCell ref="F54:G54"/>
+    <mergeCell ref="H54:I54"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="F53:G53"/>
+    <mergeCell ref="H53:I53"/>
+    <mergeCell ref="D45:E45"/>
+    <mergeCell ref="J45:K45"/>
+    <mergeCell ref="F48:G48"/>
+    <mergeCell ref="H48:I48"/>
+    <mergeCell ref="J48:K48"/>
+    <mergeCell ref="D52:E52"/>
+    <mergeCell ref="F46:G46"/>
+    <mergeCell ref="J46:K46"/>
+    <mergeCell ref="D47:E47"/>
+    <mergeCell ref="F47:G47"/>
+    <mergeCell ref="H47:I47"/>
+    <mergeCell ref="H60:I60"/>
+    <mergeCell ref="D55:E55"/>
+    <mergeCell ref="F55:G55"/>
+    <mergeCell ref="H55:I55"/>
+    <mergeCell ref="F76:G76"/>
+    <mergeCell ref="D91:E91"/>
+    <mergeCell ref="F91:G91"/>
+    <mergeCell ref="F45:G45"/>
+    <mergeCell ref="H45:I45"/>
+    <mergeCell ref="F84:G84"/>
+    <mergeCell ref="D90:E90"/>
+    <mergeCell ref="F90:G90"/>
+    <mergeCell ref="D87:E87"/>
+    <mergeCell ref="F87:G87"/>
+    <mergeCell ref="D89:E89"/>
+    <mergeCell ref="F89:G89"/>
+    <mergeCell ref="F80:G80"/>
+    <mergeCell ref="D85:E85"/>
+    <mergeCell ref="F85:G85"/>
+    <mergeCell ref="D86:E86"/>
+    <mergeCell ref="F86:G86"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="F81:G81"/>
+    <mergeCell ref="D82:E82"/>
     <mergeCell ref="D73:E73"/>
     <mergeCell ref="H66:I66"/>
     <mergeCell ref="J66:K66"/>
@@ -35394,239 +35598,21 @@
     <mergeCell ref="D56:E56"/>
     <mergeCell ref="D59:G59"/>
     <mergeCell ref="H59:I59"/>
-    <mergeCell ref="H60:I60"/>
-    <mergeCell ref="D55:E55"/>
-    <mergeCell ref="F55:G55"/>
-    <mergeCell ref="H55:I55"/>
-    <mergeCell ref="F76:G76"/>
-    <mergeCell ref="D91:E91"/>
-    <mergeCell ref="F91:G91"/>
-    <mergeCell ref="F45:G45"/>
-    <mergeCell ref="H45:I45"/>
-    <mergeCell ref="F84:G84"/>
-    <mergeCell ref="D90:E90"/>
-    <mergeCell ref="F90:G90"/>
-    <mergeCell ref="D87:E87"/>
-    <mergeCell ref="F87:G87"/>
-    <mergeCell ref="D89:E89"/>
-    <mergeCell ref="F89:G89"/>
-    <mergeCell ref="F80:G80"/>
-    <mergeCell ref="D85:E85"/>
-    <mergeCell ref="F85:G85"/>
-    <mergeCell ref="D86:E86"/>
-    <mergeCell ref="F86:G86"/>
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="F81:G81"/>
-    <mergeCell ref="D82:E82"/>
-    <mergeCell ref="D54:E54"/>
-    <mergeCell ref="F54:G54"/>
-    <mergeCell ref="H54:I54"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="F53:G53"/>
-    <mergeCell ref="H53:I53"/>
-    <mergeCell ref="D45:E45"/>
-    <mergeCell ref="J45:K45"/>
-    <mergeCell ref="F48:G48"/>
-    <mergeCell ref="H48:I48"/>
-    <mergeCell ref="J48:K48"/>
-    <mergeCell ref="D52:E52"/>
-    <mergeCell ref="F46:G46"/>
-    <mergeCell ref="J46:K46"/>
-    <mergeCell ref="D47:E47"/>
-    <mergeCell ref="F47:G47"/>
-    <mergeCell ref="H47:I47"/>
-    <mergeCell ref="A22:A37"/>
-    <mergeCell ref="A39:A56"/>
-    <mergeCell ref="A58:A73"/>
-    <mergeCell ref="A75:A91"/>
-    <mergeCell ref="D78:E78"/>
-    <mergeCell ref="F78:G78"/>
-    <mergeCell ref="F79:G79"/>
-    <mergeCell ref="D72:E72"/>
-    <mergeCell ref="F72:G72"/>
-    <mergeCell ref="H72:I72"/>
-    <mergeCell ref="F73:G73"/>
-    <mergeCell ref="J43:K43"/>
-    <mergeCell ref="D71:E71"/>
-    <mergeCell ref="F44:G44"/>
-    <mergeCell ref="H44:I44"/>
-    <mergeCell ref="D43:E43"/>
-    <mergeCell ref="F43:G43"/>
-    <mergeCell ref="D84:E84"/>
-    <mergeCell ref="D68:E68"/>
-    <mergeCell ref="F52:G52"/>
-    <mergeCell ref="B21:C21"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="C25:C27"/>
-    <mergeCell ref="C28:C35"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="C81:C89"/>
-    <mergeCell ref="C78:C80"/>
-    <mergeCell ref="C46:C54"/>
-    <mergeCell ref="C61:C63"/>
-    <mergeCell ref="C64:C69"/>
-    <mergeCell ref="B74:C74"/>
-    <mergeCell ref="B57:C57"/>
-    <mergeCell ref="C70:C71"/>
-    <mergeCell ref="C40:C41"/>
-    <mergeCell ref="C43:C45"/>
-    <mergeCell ref="G1:J2"/>
-    <mergeCell ref="A2:E4"/>
-    <mergeCell ref="G3:J3"/>
-    <mergeCell ref="G4:J4"/>
-    <mergeCell ref="C6:C7"/>
-    <mergeCell ref="C8:C10"/>
-    <mergeCell ref="H6:I6"/>
-    <mergeCell ref="D6:G6"/>
-    <mergeCell ref="D7:G7"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="J8:K8"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="A6:A20"/>
-    <mergeCell ref="C11:C20"/>
-    <mergeCell ref="J14:K14"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="J12:K12"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="I11:J11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J71:K71"/>
-    <mergeCell ref="D69:E69"/>
-    <mergeCell ref="F69:G69"/>
-    <mergeCell ref="D70:E70"/>
-    <mergeCell ref="F70:G70"/>
-    <mergeCell ref="H70:I70"/>
-    <mergeCell ref="J70:K70"/>
-    <mergeCell ref="F71:G71"/>
-    <mergeCell ref="J68:K68"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="H73:I73"/>
-    <mergeCell ref="F82:G82"/>
-    <mergeCell ref="D83:E83"/>
-    <mergeCell ref="F83:G83"/>
-    <mergeCell ref="H68:I68"/>
-    <mergeCell ref="D79:E79"/>
-    <mergeCell ref="D80:E80"/>
-    <mergeCell ref="D76:E76"/>
-    <mergeCell ref="D77:G77"/>
-    <mergeCell ref="F68:G68"/>
-    <mergeCell ref="H69:I69"/>
-    <mergeCell ref="H71:I71"/>
-    <mergeCell ref="H46:I46"/>
-    <mergeCell ref="H52:I52"/>
-    <mergeCell ref="D60:G60"/>
-    <mergeCell ref="D61:E61"/>
-    <mergeCell ref="D44:E44"/>
-    <mergeCell ref="D49:E49"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="D50:E50"/>
-    <mergeCell ref="D51:E51"/>
-    <mergeCell ref="J53:K53"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H43:I43"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H10:I10"/>
-    <mergeCell ref="D42:G42"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="I31:J31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="H28:I28"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="F28:G28"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="F36:G36"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="D41:G41"/>
-    <mergeCell ref="H41:I41"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="F19:G19"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="F20:G20"/>
-    <mergeCell ref="H20:I20"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="J15:K15"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="H23:I23"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="H24:I24"/>
-    <mergeCell ref="H17:I17"/>
-    <mergeCell ref="H36:I36"/>
-    <mergeCell ref="F99:G99"/>
-    <mergeCell ref="H25:I25"/>
-    <mergeCell ref="J25:K25"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="F26:G26"/>
-    <mergeCell ref="H26:I26"/>
-    <mergeCell ref="J26:K26"/>
-    <mergeCell ref="F25:G25"/>
-    <mergeCell ref="H62:I62"/>
-    <mergeCell ref="H63:I63"/>
-    <mergeCell ref="H51:I51"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="D40:G40"/>
-    <mergeCell ref="H40:I40"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="F35:G35"/>
-    <mergeCell ref="H35:I35"/>
-    <mergeCell ref="J35:K35"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="F64:G64"/>
-    <mergeCell ref="D48:E48"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="H42:I42"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="F66:G66"/>
-    <mergeCell ref="F51:G51"/>
-    <mergeCell ref="F62:G62"/>
-    <mergeCell ref="H12:I12"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="F15:G15"/>
-    <mergeCell ref="H15:I15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="F16:G16"/>
-    <mergeCell ref="H16:K16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="F17:G17"/>
-    <mergeCell ref="J17:K17"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="H76:H91"/>
+    <mergeCell ref="I77:J77"/>
+    <mergeCell ref="I85:J85"/>
+    <mergeCell ref="I84:J84"/>
+    <mergeCell ref="I83:J83"/>
+    <mergeCell ref="I82:J82"/>
+    <mergeCell ref="I81:J81"/>
+    <mergeCell ref="I80:J80"/>
+    <mergeCell ref="I79:J79"/>
+    <mergeCell ref="I78:J78"/>
+    <mergeCell ref="I91:J91"/>
+    <mergeCell ref="I90:J90"/>
+    <mergeCell ref="I89:J89"/>
+    <mergeCell ref="I87:J87"/>
+    <mergeCell ref="I86:J86"/>
   </mergeCells>
   <pageMargins left="0.216187305364964" right="0.14099172089019399" top="0.26" bottom="0.25" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToHeight="0" orientation="landscape" r:id="rId1"/>
@@ -35647,91 +35633,91 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="309" t="s">
+      <c r="A1" s="306" t="s">
         <v>164</v>
       </c>
-      <c r="B1" s="310"/>
-      <c r="C1" s="310"/>
-      <c r="D1" s="310"/>
-      <c r="E1" s="310"/>
-      <c r="F1" s="311"/>
+      <c r="B1" s="307"/>
+      <c r="C1" s="307"/>
+      <c r="D1" s="307"/>
+      <c r="E1" s="307"/>
+      <c r="F1" s="308"/>
     </row>
     <row r="2" spans="1:9" ht="18" x14ac:dyDescent="0.25">
-      <c r="A2" s="312" t="s">
+      <c r="A2" s="309" t="s">
         <v>164</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>46</v>
       </c>
       <c r="C2" s="3"/>
-      <c r="D2" s="125" t="s">
-        <v>275</v>
-      </c>
-      <c r="E2" s="125" t="s">
-        <v>276</v>
-      </c>
-      <c r="F2" s="126" t="s">
-        <v>277</v>
+      <c r="D2" s="321" t="s">
+        <v>165</v>
+      </c>
+      <c r="E2" s="321" t="s">
+        <v>166</v>
+      </c>
+      <c r="F2" s="322" t="s">
+        <v>167</v>
       </c>
       <c r="G2" s="5" t="s">
-        <v>333</v>
+        <v>329</v>
       </c>
       <c r="H2" s="5" t="s">
-        <v>334</v>
+        <v>330</v>
       </c>
       <c r="I2" s="5" t="s">
-        <v>335</v>
+        <v>331</v>
       </c>
     </row>
     <row r="3" spans="1:9" ht="90" x14ac:dyDescent="0.25">
-      <c r="A3" s="313"/>
+      <c r="A3" s="310"/>
       <c r="B3" s="107" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="C3" s="105"/>
       <c r="D3" s="106" t="s">
-        <v>300</v>
+        <v>296</v>
       </c>
       <c r="E3" s="106" t="s">
-        <v>299</v>
+        <v>295</v>
       </c>
       <c r="F3" s="106" t="s">
-        <v>298</v>
+        <v>294</v>
       </c>
       <c r="G3" s="106" t="s">
-        <v>297</v>
+        <v>293</v>
       </c>
       <c r="H3" s="106" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="I3" s="106" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="72" x14ac:dyDescent="0.25">
+      <c r="A4" s="310"/>
+      <c r="B4" s="107" t="s">
         <v>267</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" ht="72" x14ac:dyDescent="0.25">
-      <c r="A4" s="313"/>
-      <c r="B4" s="107" t="s">
-        <v>268</v>
       </c>
       <c r="C4" s="105"/>
       <c r="D4" s="106" t="s">
+        <v>287</v>
+      </c>
+      <c r="E4" s="106" t="s">
+        <v>288</v>
+      </c>
+      <c r="F4" s="106" t="s">
+        <v>289</v>
+      </c>
+      <c r="G4" s="106" t="s">
+        <v>290</v>
+      </c>
+      <c r="H4" s="106" t="s">
         <v>291</v>
       </c>
-      <c r="E4" s="106" t="s">
-        <v>292</v>
-      </c>
-      <c r="F4" s="106" t="s">
-        <v>293</v>
-      </c>
-      <c r="G4" s="106" t="s">
-        <v>294</v>
-      </c>
-      <c r="H4" s="106" t="s">
-        <v>295</v>
-      </c>
     </row>
     <row r="5" spans="1:9" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A5" s="314"/>
+      <c r="A5" s="311"/>
       <c r="B5" s="6" t="s">
         <v>9</v>
       </c>
@@ -35743,7 +35729,7 @@
       <c r="F5" s="9"/>
     </row>
     <row r="6" spans="1:9" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A6" s="314"/>
+      <c r="A6" s="311"/>
       <c r="B6" s="6" t="s">
         <v>13</v>
       </c>
@@ -35752,12 +35738,12 @@
         <v>169</v>
       </c>
       <c r="E6" s="8" t="s">
-        <v>336</v>
+        <v>332</v>
       </c>
       <c r="F6" s="10"/>
     </row>
     <row r="7" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A7" s="314"/>
+      <c r="A7" s="311"/>
       <c r="B7" s="6" t="s">
         <v>15</v>
       </c>
@@ -35769,15 +35755,15 @@
         <v>171</v>
       </c>
       <c r="F7" s="9" t="s">
-        <v>337</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A8" s="314"/>
+      <c r="A8" s="311"/>
       <c r="B8" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="316"/>
+      <c r="C8" s="313"/>
       <c r="D8" s="8" t="s">
         <v>172</v>
       </c>
@@ -35789,11 +35775,11 @@
       </c>
     </row>
     <row r="9" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A9" s="314"/>
+      <c r="A9" s="311"/>
       <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="317"/>
+      <c r="C9" s="314"/>
       <c r="D9" s="8" t="s">
         <v>175</v>
       </c>
@@ -35803,11 +35789,11 @@
       <c r="F9" s="11"/>
     </row>
     <row r="10" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A10" s="314"/>
+      <c r="A10" s="311"/>
       <c r="B10" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="317"/>
+      <c r="C10" s="314"/>
       <c r="D10" s="8" t="s">
         <v>177</v>
       </c>
@@ -35819,11 +35805,11 @@
       </c>
     </row>
     <row r="11" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A11" s="314"/>
+      <c r="A11" s="311"/>
       <c r="B11" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="C11" s="317"/>
+      <c r="C11" s="314"/>
       <c r="D11" s="8" t="s">
         <v>180</v>
       </c>
@@ -35835,87 +35821,87 @@
       </c>
     </row>
     <row r="12" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A12" s="314"/>
+      <c r="A12" s="311"/>
       <c r="B12" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="315"/>
+      <c r="D12" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="C12" s="318"/>
-      <c r="D12" s="8" t="s">
+      <c r="E12" s="8" t="s">
         <v>184</v>
       </c>
-      <c r="E12" s="8" t="s">
+      <c r="F12" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="F12" s="9" t="s">
+    </row>
+    <row r="13" spans="1:9" ht="74.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="311"/>
+      <c r="B13" s="6" t="s">
         <v>186</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" ht="74.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="314"/>
-      <c r="B13" s="6" t="s">
-        <v>187</v>
       </c>
       <c r="C13" s="13"/>
       <c r="E13" s="8" t="s">
+        <v>187</v>
+      </c>
+      <c r="F13" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="F13" s="9" t="s">
-        <v>189</v>
-      </c>
     </row>
     <row r="14" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A14" s="314"/>
+      <c r="A14" s="311"/>
       <c r="B14" s="6" t="s">
         <v>32</v>
       </c>
       <c r="C14" s="13"/>
       <c r="D14" s="2"/>
       <c r="E14" s="8" t="s">
+        <v>189</v>
+      </c>
+      <c r="F14" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="F14" s="12" t="s">
-        <v>191</v>
-      </c>
     </row>
     <row r="15" spans="1:9" ht="66" x14ac:dyDescent="0.25">
-      <c r="A15" s="314"/>
+      <c r="A15" s="311"/>
       <c r="B15" s="6" t="s">
         <v>35</v>
       </c>
       <c r="C15" s="14"/>
       <c r="D15" s="15"/>
       <c r="E15" s="8" t="s">
-        <v>340</v>
+        <v>336</v>
       </c>
       <c r="F15" s="9" t="s">
-        <v>341</v>
+        <v>337</v>
       </c>
     </row>
     <row r="16" spans="1:9" ht="57" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="315"/>
+      <c r="A16" s="312"/>
       <c r="B16" s="6" t="s">
         <v>39</v>
       </c>
       <c r="C16" s="16"/>
       <c r="D16" s="17"/>
       <c r="E16" s="17" t="s">
+        <v>191</v>
+      </c>
+      <c r="F16" s="18"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A17" s="316" t="s">
         <v>192</v>
       </c>
-      <c r="F16" s="18"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A17" s="319" t="s">
-        <v>193</v>
-      </c>
-      <c r="B17" s="320"/>
-      <c r="C17" s="320"/>
-      <c r="D17" s="320"/>
-      <c r="E17" s="320"/>
-      <c r="F17" s="321"/>
+      <c r="B17" s="317"/>
+      <c r="C17" s="317"/>
+      <c r="D17" s="317"/>
+      <c r="E17" s="317"/>
+      <c r="F17" s="318"/>
     </row>
     <row r="18" spans="1:6" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="312" t="s">
-        <v>193</v>
+      <c r="A18" s="309" t="s">
+        <v>192</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>46</v>
@@ -35932,107 +35918,107 @@
       </c>
     </row>
     <row r="19" spans="1:6" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A19" s="314"/>
+      <c r="A19" s="311"/>
       <c r="B19" s="7" t="s">
         <v>13</v>
       </c>
       <c r="C19" s="7"/>
       <c r="D19" s="1"/>
       <c r="E19" s="8" t="s">
-        <v>338</v>
+        <v>334</v>
       </c>
       <c r="F19" s="19"/>
     </row>
     <row r="20" spans="1:6" ht="49.5" x14ac:dyDescent="0.25">
-      <c r="A20" s="314"/>
+      <c r="A20" s="311"/>
       <c r="B20" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="323"/>
+      <c r="C20" s="320"/>
       <c r="D20" s="8"/>
       <c r="E20" s="8" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="F20" s="10"/>
     </row>
     <row r="21" spans="1:6" ht="66" x14ac:dyDescent="0.25">
-      <c r="A21" s="314"/>
+      <c r="A21" s="311"/>
       <c r="B21" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="317"/>
+      <c r="C21" s="314"/>
       <c r="D21" s="8" t="s">
+        <v>194</v>
+      </c>
+      <c r="E21" s="8" t="s">
         <v>195</v>
       </c>
-      <c r="E21" s="8" t="s">
+      <c r="F21" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="F21" s="9" t="s">
-        <v>197</v>
-      </c>
     </row>
     <row r="22" spans="1:6" ht="66" x14ac:dyDescent="0.25">
-      <c r="A22" s="314"/>
+      <c r="A22" s="311"/>
       <c r="B22" s="7" t="s">
         <v>25</v>
       </c>
-      <c r="C22" s="317"/>
+      <c r="C22" s="314"/>
       <c r="D22" s="8" t="s">
+        <v>197</v>
+      </c>
+      <c r="E22" s="8" t="s">
         <v>198</v>
       </c>
-      <c r="E22" s="8" t="s">
+      <c r="F22" s="9" t="s">
         <v>199</v>
       </c>
-      <c r="F22" s="9" t="s">
-        <v>200</v>
-      </c>
     </row>
     <row r="23" spans="1:6" ht="66" x14ac:dyDescent="0.25">
-      <c r="A23" s="314"/>
+      <c r="A23" s="311"/>
       <c r="B23" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C23" s="318"/>
+      <c r="C23" s="315"/>
       <c r="D23" s="8" t="s">
-        <v>339</v>
+        <v>335</v>
       </c>
       <c r="E23" s="8" t="s">
-        <v>342</v>
+        <v>338</v>
       </c>
       <c r="F23" s="9" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="24" spans="1:6" ht="66" x14ac:dyDescent="0.25">
-      <c r="A24" s="314"/>
+      <c r="A24" s="311"/>
       <c r="B24" s="7" t="s">
         <v>32</v>
       </c>
       <c r="C24" s="7"/>
       <c r="D24" s="8" t="s">
-        <v>343</v>
+        <v>339</v>
       </c>
       <c r="E24" s="8" t="s">
+        <v>201</v>
+      </c>
+      <c r="F24" s="9" t="s">
         <v>202</v>
       </c>
-      <c r="F24" s="9" t="s">
-        <v>203</v>
-      </c>
     </row>
     <row r="25" spans="1:6" ht="78" x14ac:dyDescent="0.25">
-      <c r="A25" s="322"/>
+      <c r="A25" s="319"/>
       <c r="B25" s="7" t="s">
         <v>35</v>
       </c>
       <c r="C25" s="7"/>
       <c r="D25" s="20" t="s">
+        <v>203</v>
+      </c>
+      <c r="E25" s="20" t="s">
         <v>204</v>
       </c>
-      <c r="E25" s="20" t="s">
+      <c r="F25" s="9" t="s">
         <v>205</v>
-      </c>
-      <c r="F25" s="9" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="26" spans="1:6" ht="78" x14ac:dyDescent="0.25">
@@ -36042,27 +36028,27 @@
       </c>
       <c r="C26" s="22"/>
       <c r="D26" s="23" t="s">
+        <v>206</v>
+      </c>
+      <c r="E26" s="23" t="s">
         <v>207</v>
-      </c>
-      <c r="E26" s="23" t="s">
-        <v>208</v>
       </c>
       <c r="F26" s="24"/>
     </row>
     <row r="27" spans="1:6" ht="78" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
       <c r="B27" s="26" t="s">
-        <v>183</v>
+        <v>42</v>
       </c>
       <c r="C27" s="26"/>
       <c r="D27" s="27" t="s">
+        <v>208</v>
+      </c>
+      <c r="E27" s="17" t="s">
         <v>209</v>
       </c>
-      <c r="E27" s="17" t="s">
+      <c r="F27" s="18" t="s">
         <v>210</v>
-      </c>
-      <c r="F27" s="18" t="s">
-        <v>211</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>